<commit_message>
added and fixed these things
</commit_message>
<xml_diff>
--- a/script2/input/ampq.xlsx
+++ b/script2/input/ampq.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Mój dysk\AMPQ\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44FABF82-6F9B-4700-8B3D-13E71C0EA91C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3361760-1272-484A-A4B8-28875E0E8B47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3465E9D8-2616-4A3B-901D-12D504620602}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="319" uniqueCount="162">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="306" uniqueCount="155">
   <si>
     <t>QTY</t>
   </si>
@@ -59,9 +59,6 @@
     <t>(in stock)</t>
   </si>
   <si>
-    <t>(in stock, EXW)</t>
-  </si>
-  <si>
     <t>Xiaomi Sound Pocket 5W Pink S28H-GL QBH4380GL</t>
   </si>
   <si>
@@ -74,12 +71,6 @@
     <t>Philips Lumea Prestige IPL 8000 BRI940/00</t>
   </si>
   <si>
-    <t>Xiaomi Robot Vacuum S20 White EU BHR8629EU</t>
-  </si>
-  <si>
-    <t>Remington Shine Therapy Pro S9300</t>
-  </si>
-  <si>
     <t>Samsung Powerbank Battery Pack 25W 10.000 mAh EB-P3400XUEGEU</t>
   </si>
   <si>
@@ -89,9 +80,6 @@
     <t>Xiaomi Toaster Black BHR8811EU</t>
   </si>
   <si>
-    <t>Xiaomi Handheld Steam Iron white BHR9034EU</t>
-  </si>
-  <si>
     <t>Ninja Air Fryer XL 9,5L SL451EU</t>
   </si>
   <si>
@@ -116,15 +104,9 @@
     <t>Xiaomi Redmi Note 15 4G NFC DS 8/256GB Midnight Black MZB0M8FEU</t>
   </si>
   <si>
-    <t>Xiaomi Redmi Note 15 4G NFC DS 8/256GB Glacier Blue MZB0MOIEU</t>
-  </si>
-  <si>
     <t>Xiaomi Redmi Pad 2 Pro WIFI 6/128GB Silver VHU6253EU</t>
   </si>
   <si>
-    <t>Ninja Luxe Café Essential ES501EU</t>
-  </si>
-  <si>
     <t>Ninja Foodi Power Nutri CB100EU</t>
   </si>
   <si>
@@ -191,15 +173,9 @@
     <t>Realme SUPERVOOC 120W Power Adapter white</t>
   </si>
   <si>
-    <t>Apple iPhone 17 256GB Sage MG6N4HX/A</t>
-  </si>
-  <si>
     <t>Realme Buds Air 8 Gray EU</t>
   </si>
   <si>
-    <t>Apple iPhone 17 256GB Black MG6J4HN/A</t>
-  </si>
-  <si>
     <t>Apple iPhone 17 256GB Lavender MG6M4HN/A</t>
   </si>
   <si>
@@ -218,9 +194,6 @@
     <t>Karcher WV 5 Plus N White EU 1.633-701.0</t>
   </si>
   <si>
-    <t>Xiaomi Redmi Note 15 Pro 4G 8/256GB Black MZB0LYMEU</t>
-  </si>
-  <si>
     <t>Logitech Racing Set G29 PS3/PS4/PS5 941-000112</t>
   </si>
   <si>
@@ -230,9 +203,6 @@
     <t>Xiaomi Electric Scooter 4 Ultra BHR6151DE</t>
   </si>
   <si>
-    <t>Apple iPhone 16 128GB White MYE93HN/A</t>
-  </si>
-  <si>
     <t>Dyson Wash G1 WR01 Cordless Vacuum Blue/Black EU 486236-01</t>
   </si>
   <si>
@@ -248,15 +218,9 @@
     <t>Tefal Ultragliss Plus Iron Blue FV6812E0</t>
   </si>
   <si>
-    <t>Tefal Digital Kettle BLK KI831E10</t>
-  </si>
-  <si>
     <t>Tefal Express Steam Iron Claret FV2835E0</t>
   </si>
   <si>
-    <t>Xiaomi Redmi Note 15 Pro+ 5G 8/256GB Mocha Brown MZB0MIGEU</t>
-  </si>
-  <si>
     <t>Xiaomi Redmi 15C 4G 8/256GB Midnight Black MZB0KTPEU</t>
   </si>
   <si>
@@ -266,9 +230,6 @@
     <t>Xiaomi Redmi 15C 4G 8/256GB Mint Green MZB0LBVEU</t>
   </si>
   <si>
-    <t>Xiaomi Smart Air Purifier 4 compact BHR5860EU</t>
-  </si>
-  <si>
     <t>Logitech Mouse M240 Silent Pink 910-007121</t>
   </si>
   <si>
@@ -314,18 +275,9 @@
     <t>Xiaomi 33W Power Bank 10000mAh Integrated Cable BHR9333GL</t>
   </si>
   <si>
-    <t>Xiaomi 33W Power Bank 20000mAh Integrated Cable Tan GL BHR8851GL</t>
-  </si>
-  <si>
     <t>Xiaomi 67W Power Bank 20000mAh Integrated Cable Tan BHR08O7GL</t>
   </si>
   <si>
-    <t>OnePlus 15 16/512GB Black</t>
-  </si>
-  <si>
-    <t>OnePlus 15 16/512GB Sand Storm</t>
-  </si>
-  <si>
     <t>Realme 16 Pro+ 5G 12/512GB Grey EU</t>
   </si>
   <si>
@@ -350,9 +302,6 @@
     <t>Tefal Ultimate Power Pro Black/Copper FV9E50E0</t>
   </si>
   <si>
-    <t>Tefal Ulitmate Pure Gold FV9852E0</t>
-  </si>
-  <si>
     <t>Tefal SMART PROTECT PLUS Blue/Silver FV6872E0</t>
   </si>
   <si>
@@ -368,15 +317,9 @@
     <t>Tefal Express Steam Iron Generator White&amp;Black SV8130E0</t>
   </si>
   <si>
-    <t>Tefal Ulitmate Pure Gold/Black FV9845E0</t>
-  </si>
-  <si>
     <t>Tefal Easygliss Plus 2 FV5718E0</t>
   </si>
   <si>
-    <t>Tefal Ultimate Pure Black/Blue FV9848E0</t>
-  </si>
-  <si>
     <t>Karcher SC 3 EasyFix EU 1.513-650.0</t>
   </si>
   <si>
@@ -389,12 +332,6 @@
     <t>Karcher WV 2 Premium 1.633-426.0</t>
   </si>
   <si>
-    <t>Apple iPhone 15 128GB Blue MTP43HN/A</t>
-  </si>
-  <si>
-    <t>Xiaomi Redmi A5 4G 3/64GB Midnight Black MZB0JSEEU</t>
-  </si>
-  <si>
     <t>Xiaomi Redmi A5 4G 3/64GB Sandy Gold MZB0JTEEU</t>
   </si>
   <si>
@@ -422,106 +359,148 @@
     <t>Xiaomi Redmi Note 15 5G 8/256GB Black MZB0LWMEU</t>
   </si>
   <si>
-    <t>Xiaomi Redmi Note 15 5G 8/256GB Glacier Blue MZB0LWKEU</t>
-  </si>
-  <si>
-    <t>Xiaomi Redmi Note 15 Pro+ 5G 8/256GB Glacier Blue MZB0MI3EU</t>
-  </si>
-  <si>
-    <t>Xiaomi Poco X8 Pro Max 5G DS 12/256GB White MZB0NBSEU</t>
-  </si>
-  <si>
-    <t>Xiaomi Poco X8 Pro Max 5G DS 12/512GB Black MZB0NBWEU</t>
-  </si>
-  <si>
     <t>(incoming 1-2 days)</t>
   </si>
   <si>
+    <t>Babyliss Curling iron C338E</t>
+  </si>
+  <si>
+    <t>Babyliss Hair dryer brush AS962E</t>
+  </si>
+  <si>
+    <t>Babyliss Hair dryer brush AS960E</t>
+  </si>
+  <si>
+    <t>JBL PartyBox Encore 2 JBLPBENCORE2EP</t>
+  </si>
+  <si>
+    <t>JBL PartyBox Encore Essential 2 JBLPBENCOREESS2EP</t>
+  </si>
+  <si>
+    <t>Karcher Electric Mop EWM 2 1.056-310.0</t>
+  </si>
+  <si>
+    <t>Oral-B Vitality D103 Pro Box LilacViolet 426967</t>
+  </si>
+  <si>
+    <t>Oral-B Vitality D103 Pro Box Blue 446392</t>
+  </si>
+  <si>
+    <t>Oral-B Vitality Pro Duo Black/Lilac Violet D103</t>
+  </si>
+  <si>
+    <t>Oral-B ELEC TB PRO 1 BLACK TRAVEL CASE 914170</t>
+  </si>
+  <si>
+    <t>Oral-B ELEC TB PRO 1 PINK TRAVEL CASE 3216721</t>
+  </si>
+  <si>
+    <t>Oral-B IO2 Duo Pack Xmas Edition</t>
+  </si>
+  <si>
+    <t>Oral-B ELEC TB VITALITY PRO FROZEN + TRAVEL CASE</t>
+  </si>
+  <si>
+    <t>Russell Hobbs Air Fryer 5L 1650 W Black 26510-56</t>
+  </si>
+  <si>
+    <t>Tefal Virtuo Navy Blue FV1713</t>
+  </si>
+  <si>
+    <t>Bosch Toaster Black TAT6A513</t>
+  </si>
+  <si>
+    <t>Philips Hair Dryer 1600 W Black BHD302/10</t>
+  </si>
+  <si>
+    <t>Xiaomi Poco Pad M1 8/256GB Grey VHU6302EU</t>
+  </si>
+  <si>
+    <t>Google Pixel 10a 8/128GB Black GA09561-GB</t>
+  </si>
+  <si>
+    <t>CHiQ Monitor 27" 27F650R</t>
+  </si>
+  <si>
+    <t>Ecovacs Winbot cleaning solution 230ml W-SO01-0004</t>
+  </si>
+  <si>
+    <t>Ecovacs Winbot W2 Pro Omni WG851-11EDR</t>
+  </si>
+  <si>
+    <t>Ecovacs Winbot W2 Pro WG852-11EDR</t>
+  </si>
+  <si>
+    <t>Huawei Watch Fit 4 Seiya-B19F White Fluoroelastomer Strap 55020EYL</t>
+  </si>
+  <si>
+    <t>Huawei Watch GT 5 Vili-B19F Black Fluoroelastomer Strap 55020DKM</t>
+  </si>
+  <si>
+    <t>Huawei Watch GT 5 Jana-B19L White Composite Leather Strap 55020DJT</t>
+  </si>
+  <si>
+    <t>Huawei Watch GT 5 Vili-B19W Blue Woven Strap 55020DKH</t>
+  </si>
+  <si>
+    <t>Huawei Watch GT 5 Jana-B19M Gold Milanese Strap 55020DJQ</t>
+  </si>
+  <si>
+    <t>Huawei Watch GT 5 Pro Vili-B29F Black Fluoroelastomer Strap 55020DKD</t>
+  </si>
+  <si>
+    <t>Huawei Watch 5 LTE 46mm Rates-L19F Black 55020EWB</t>
+  </si>
+  <si>
+    <t>Huawei Watch GT 6 41MM Konsu-B19M Gold 55020FTP</t>
+  </si>
+  <si>
+    <t>Huawei Watch GT 6 Pro 46MM Atum-B29M Titanium 55020FTT</t>
+  </si>
+  <si>
+    <t>Samsung SmartTag2 Black EI-T5600BBEGEU</t>
+  </si>
+  <si>
+    <t>Samsung SmartTag2 White EI-T5600BWEGEU</t>
+  </si>
+  <si>
+    <t>Samsung Galaxy Fit3 Gray SM-R390NZAAMEA</t>
+  </si>
+  <si>
+    <t>Samsung Galaxy Fit3 Pink Gold SM-R390NZDAEUE</t>
+  </si>
+  <si>
+    <t>Samsung Galaxy Fit3 Silver SM-R390NZSAEUE</t>
+  </si>
+  <si>
+    <t>(in stock EXW)</t>
+  </si>
+  <si>
+    <t>Xiaomi Robot Vacuum S40 BHR084AEU</t>
+  </si>
+  <si>
+    <t>(incoming 12.05)</t>
+  </si>
+  <si>
     <t>Apple Pencil 2nd Generation White MXN43ZM/A</t>
   </si>
   <si>
-    <t>Babyliss Curling iron C338E</t>
-  </si>
-  <si>
-    <t>Babyliss Curling iron C451E</t>
-  </si>
-  <si>
-    <t>Babyliss Hair dryer brush AS962E</t>
-  </si>
-  <si>
-    <t>Babyliss Hair dryer brush AS960E</t>
-  </si>
-  <si>
-    <t>JBL PartyBox Encore 2 JBLPBENCORE2EP</t>
-  </si>
-  <si>
-    <t>JBL PartyBox Encore Essential 2 JBLPBENCOREESS2EP</t>
-  </si>
-  <si>
-    <t>JBL Tune 530BT Beige JBLT530BTBEGEU</t>
-  </si>
-  <si>
-    <t>JBL Tune 530BT Black JBLT530BTBLKEU</t>
-  </si>
-  <si>
-    <t>JBL Tune 530BT Lavender JBLT530BTLAVEU</t>
-  </si>
-  <si>
-    <t>Karcher Electric Mop EWM 2 1.056-310.0</t>
-  </si>
-  <si>
-    <t>Oral-B Vitality D103 Pro Box LilacViolet 426967</t>
-  </si>
-  <si>
-    <t>Oral-B Vitality D103 Pro Box Blue 446392</t>
-  </si>
-  <si>
-    <t>Oral-B Vitality Pro Duo Black/Lilac Violet D103</t>
-  </si>
-  <si>
-    <t>Oral-B ELEC TB PRO 1 BLACK TRAVEL CASE 914170</t>
-  </si>
-  <si>
-    <t>Oral-B ELEC TB PRO 1 PINK TRAVEL CASE 3216721</t>
-  </si>
-  <si>
-    <t>Oral-B IO2 Duo Pack Xmas Edition</t>
-  </si>
-  <si>
-    <t>Oral-B ELEC TB VITALITY PRO FROZEN + TRAVEL CASE</t>
-  </si>
-  <si>
-    <t>Orall-B ELEC TB VITALITY PRO LION KING + TRAVEL CASE</t>
-  </si>
-  <si>
-    <t>Russell Hobbs Air Fryer 5L 1650 W Black 26510-56</t>
-  </si>
-  <si>
-    <t>Tefal Virtuo Navy Blue FV1713</t>
-  </si>
-  <si>
-    <t>Vileda Sun-Rise Premium 50m</t>
-  </si>
-  <si>
-    <t>Bosch Toaster Black TAT6A513</t>
-  </si>
-  <si>
-    <t>Philips Hair Dryer 1600 W Black BHD302/10</t>
-  </si>
-  <si>
-    <t>Samsung Tab A11+ 11" WIFI 6/128GB Grey SM-X230NZAREUE</t>
-  </si>
-  <si>
-    <t>Xiaomi Poco Pad M1 8/256GB Grey VHU6302EU</t>
-  </si>
-  <si>
-    <t>Babyliss Hair clipper E976E</t>
-  </si>
-  <si>
-    <t>c</t>
-  </si>
-  <si>
-    <t>(incoming 05.05)</t>
+    <t>Samsung A16 DS 4/128GB Black SM-A165FZKBEUE</t>
+  </si>
+  <si>
+    <t>Samsung A57 8/256GB 5G DS Navy SM-A576BDBDEUE</t>
+  </si>
+  <si>
+    <t>Samsung S26 DS 12/256GB Black SM-S942BZKGEUE</t>
+  </si>
+  <si>
+    <t>Samsung Galaxy S26 Ultra 512GB Black SM-S948BZKGEUE</t>
+  </si>
+  <si>
+    <t>Samsung Tab A11+ 5G 6GB/128GB 11" Grey SM-X236BZAREUE</t>
+  </si>
+  <si>
+    <t>Oral-B ELEC TB VITALITY PRO LION KING + TRAVEL CASE</t>
   </si>
 </sst>
 </file>
@@ -911,7 +890,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2A360796-7343-4130-90EE-C427191F85B0}">
-  <dimension ref="A1:F152"/>
+  <dimension ref="A1:F146"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" bestFit="1" customWidth="1"/>
@@ -944,13 +923,13 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B2" t="s">
-        <v>80</v>
+        <v>67</v>
       </c>
       <c r="C2" t="str">
-        <f t="shared" ref="C2:C62" si="0">MID(B2,FIND("@",SUBSTITUTE(B2," ","@",LEN(B2)-LEN(SUBSTITUTE(B2," ",""))))+1,LEN(B2))</f>
+        <f t="shared" ref="C2:C61" si="0">MID(B2,FIND("@",SUBSTITUTE(B2," ","@",LEN(B2)-LEN(SUBSTITUTE(B2," ",""))))+1,LEN(B2))</f>
         <v>MG8H4HX/A</v>
       </c>
       <c r="D2" s="3">
@@ -965,10 +944,10 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="B3" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="C3" t="str">
         <f t="shared" si="0"/>
@@ -978,7 +957,7 @@
         <v>195950644050</v>
       </c>
       <c r="E3">
-        <v>719</v>
+        <v>717</v>
       </c>
       <c r="F3" t="s">
         <v>6</v>
@@ -986,10 +965,10 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="B4" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="C4" t="str">
         <f t="shared" si="0"/>
@@ -999,7 +978,7 @@
         <v>195950643855</v>
       </c>
       <c r="E4">
-        <v>719</v>
+        <v>717</v>
       </c>
       <c r="F4" t="s">
         <v>6</v>
@@ -1007,20 +986,20 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="B5" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="C5" t="str">
         <f t="shared" si="0"/>
-        <v>MG6N4HX/A</v>
+        <v>MG6M4HN/A</v>
       </c>
       <c r="D5" s="3">
-        <v>195950644258</v>
+        <v>195950644043</v>
       </c>
       <c r="E5">
-        <v>719</v>
+        <v>695</v>
       </c>
       <c r="F5" t="s">
         <v>6</v>
@@ -1028,17 +1007,17 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="B6" t="s">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="C6" t="str">
         <f t="shared" si="0"/>
-        <v>MG6J4HN/A</v>
+        <v>MG6L4HN/A</v>
       </c>
       <c r="D6" s="3">
-        <v>195950643442</v>
+        <v>195950643848</v>
       </c>
       <c r="E6">
         <v>695</v>
@@ -1052,14 +1031,14 @@
         <v>20</v>
       </c>
       <c r="B7" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="C7" t="str">
         <f t="shared" si="0"/>
-        <v>MG6M4HN/A</v>
+        <v>MG6K4HN/A</v>
       </c>
       <c r="D7" s="3">
-        <v>195950644043</v>
+        <v>195950643640</v>
       </c>
       <c r="E7">
         <v>695</v>
@@ -1070,20 +1049,20 @@
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="B8" t="s">
-        <v>55</v>
+        <v>73</v>
       </c>
       <c r="C8" t="str">
         <f t="shared" si="0"/>
-        <v>MG6L4HN/A</v>
+        <v>MYE73HN/A</v>
       </c>
       <c r="D8" s="3">
-        <v>195950643848</v>
+        <v>195949821837</v>
       </c>
       <c r="E8">
-        <v>695</v>
+        <v>579</v>
       </c>
       <c r="F8" t="s">
         <v>6</v>
@@ -1091,20 +1070,20 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="B9" t="s">
-        <v>56</v>
+        <v>74</v>
       </c>
       <c r="C9" t="str">
         <f t="shared" si="0"/>
-        <v>MG6K4HN/A</v>
+        <v>MYED3HN/A</v>
       </c>
       <c r="D9" s="3">
-        <v>195950643640</v>
+        <v>195949822551</v>
       </c>
       <c r="E9">
-        <v>695</v>
+        <v>579</v>
       </c>
       <c r="F9" t="s">
         <v>6</v>
@@ -1112,20 +1091,20 @@
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10">
-        <v>40</v>
+        <v>195</v>
       </c>
       <c r="B10" t="s">
-        <v>86</v>
+        <v>148</v>
       </c>
       <c r="C10" t="str">
         <f t="shared" si="0"/>
-        <v>MYE73HN/A</v>
+        <v>MXN43ZM/A</v>
       </c>
       <c r="D10" s="3">
-        <v>195949821837</v>
+        <v>195949690457</v>
       </c>
       <c r="E10">
-        <v>579</v>
+        <v>58</v>
       </c>
       <c r="F10" t="s">
         <v>6</v>
@@ -1133,20 +1112,20 @@
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="B11" t="s">
-        <v>87</v>
+        <v>126</v>
       </c>
       <c r="C11" t="str">
         <f t="shared" si="0"/>
-        <v>MYED3HN/A</v>
+        <v>GA09561-GB</v>
       </c>
       <c r="D11" s="3">
-        <v>195949822551</v>
+        <v>840353949737</v>
       </c>
       <c r="E11">
-        <v>579</v>
+        <v>359</v>
       </c>
       <c r="F11" t="s">
         <v>6</v>
@@ -1154,20 +1133,19 @@
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12">
-        <v>10</v>
+        <v>200</v>
       </c>
       <c r="B12" t="s">
-        <v>64</v>
-      </c>
-      <c r="C12" t="str">
-        <f t="shared" si="0"/>
-        <v>MYE93HN/A</v>
+        <v>83</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>18</v>
       </c>
       <c r="D12" s="3">
-        <v>195949822018</v>
+        <v>6941764461062</v>
       </c>
       <c r="E12">
-        <v>579</v>
+        <v>292</v>
       </c>
       <c r="F12" t="s">
         <v>6</v>
@@ -1175,20 +1153,19 @@
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13">
-        <v>5</v>
+        <v>35</v>
       </c>
       <c r="B13" t="s">
-        <v>117</v>
-      </c>
-      <c r="C13" t="str">
-        <f t="shared" si="0"/>
-        <v>MTP43HN/A</v>
+        <v>80</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>18</v>
       </c>
       <c r="D13" s="3">
-        <v>195949036477</v>
+        <v>6941764482890</v>
       </c>
       <c r="E13">
-        <v>495</v>
+        <v>355</v>
       </c>
       <c r="F13" t="s">
         <v>6</v>
@@ -1196,60 +1173,62 @@
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14">
-        <v>190</v>
+        <v>500</v>
       </c>
       <c r="B14" t="s">
-        <v>133</v>
+        <v>149</v>
       </c>
       <c r="C14" t="str">
         <f t="shared" si="0"/>
-        <v>MXN43ZM/A</v>
+        <v>SM-A165FZKBEUE</v>
       </c>
       <c r="D14" s="3">
-        <v>190198893376</v>
+        <v>8806095822334</v>
       </c>
       <c r="E14">
-        <v>57</v>
+        <v>92</v>
       </c>
       <c r="F14" t="s">
-        <v>6</v>
+        <v>147</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15">
-        <v>40</v>
+        <v>100</v>
       </c>
       <c r="B15" t="s">
-        <v>94</v>
-      </c>
-      <c r="C15" s="5" t="s">
-        <v>22</v>
+        <v>150</v>
+      </c>
+      <c r="C15" t="str">
+        <f t="shared" si="0"/>
+        <v>SM-A576BDBDEUE</v>
       </c>
       <c r="D15" s="3">
-        <v>6921815630357</v>
+        <v>8806099028244</v>
       </c>
       <c r="E15">
-        <v>665</v>
+        <v>295</v>
       </c>
       <c r="F15" t="s">
-        <v>6</v>
+        <v>107</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16">
-        <v>15</v>
+        <v>75</v>
       </c>
       <c r="B16" t="s">
-        <v>95</v>
-      </c>
-      <c r="C16" s="5" t="s">
-        <v>22</v>
+        <v>75</v>
+      </c>
+      <c r="C16" t="str">
+        <f t="shared" si="0"/>
+        <v>SM-S931BZKDEUE</v>
       </c>
       <c r="D16" s="3">
-        <v>6921815630364</v>
+        <v>8806095815534</v>
       </c>
       <c r="E16">
-        <v>665</v>
+        <v>490</v>
       </c>
       <c r="F16" t="s">
         <v>6</v>
@@ -1257,60 +1236,62 @@
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17">
-        <v>200</v>
+        <v>100</v>
       </c>
       <c r="B17" t="s">
-        <v>99</v>
-      </c>
-      <c r="C17" s="5" t="s">
-        <v>22</v>
+        <v>75</v>
+      </c>
+      <c r="C17" t="str">
+        <f t="shared" si="0"/>
+        <v>SM-S931BZKDEUE</v>
       </c>
       <c r="D17" s="3">
-        <v>6941764461062</v>
+        <v>8806095815534</v>
       </c>
       <c r="E17">
-        <v>299</v>
+        <v>490</v>
       </c>
       <c r="F17" t="s">
-        <v>6</v>
+        <v>107</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="B18" t="s">
-        <v>96</v>
-      </c>
-      <c r="C18" s="5" t="s">
-        <v>22</v>
+        <v>151</v>
+      </c>
+      <c r="C18" t="str">
+        <f t="shared" si="0"/>
+        <v>SM-S942BZKGEUE</v>
       </c>
       <c r="D18" s="3">
-        <v>6941764482890</v>
+        <v>8806097827467</v>
       </c>
       <c r="E18">
-        <v>359</v>
+        <v>529</v>
       </c>
       <c r="F18" t="s">
-        <v>6</v>
+        <v>107</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19">
-        <v>75</v>
+        <v>20</v>
       </c>
       <c r="B19" t="s">
-        <v>88</v>
+        <v>19</v>
       </c>
       <c r="C19" t="str">
         <f t="shared" si="0"/>
-        <v>SM-S931BZKDEUE</v>
+        <v>SM-S942BZKHEUE</v>
       </c>
       <c r="D19" s="3">
-        <v>8806095815534</v>
+        <v>8806097827405</v>
       </c>
       <c r="E19">
-        <v>509</v>
+        <v>625</v>
       </c>
       <c r="F19" t="s">
         <v>6</v>
@@ -1318,62 +1299,62 @@
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20">
-        <v>35</v>
+        <v>100</v>
       </c>
       <c r="B20" t="s">
-        <v>23</v>
+        <v>152</v>
       </c>
       <c r="C20" t="str">
         <f t="shared" si="0"/>
-        <v>SM-S942BZKHEUE</v>
+        <v>SM-S948BZKGEUE</v>
       </c>
       <c r="D20" s="3">
-        <v>8806097827405</v>
+        <v>8806097827177</v>
       </c>
       <c r="E20">
-        <v>645</v>
+        <v>879</v>
       </c>
       <c r="F20" t="s">
-        <v>6</v>
+        <v>107</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21">
-        <v>300</v>
+        <v>120</v>
       </c>
       <c r="B21" t="s">
-        <v>157</v>
+        <v>153</v>
       </c>
       <c r="C21" t="str">
         <f t="shared" si="0"/>
-        <v>SM-X230NZAREUE</v>
+        <v>SM-X236BZAREUE</v>
       </c>
       <c r="D21" s="3">
-        <v>8806097855019</v>
+        <v>8806097854821</v>
       </c>
       <c r="E21">
-        <v>151</v>
+        <v>179</v>
       </c>
       <c r="F21" t="s">
-        <v>6</v>
+        <v>107</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22">
-        <v>5</v>
+        <v>100</v>
       </c>
       <c r="B22" t="s">
-        <v>130</v>
+        <v>98</v>
       </c>
       <c r="C22" t="str">
         <f t="shared" si="0"/>
-        <v>MZB0NBSEU</v>
+        <v>MZB0JTEEU</v>
       </c>
       <c r="D22" s="3">
-        <v>6932554496913</v>
+        <v>6932554425432</v>
       </c>
       <c r="E22">
-        <v>330</v>
+        <v>67</v>
       </c>
       <c r="F22" t="s">
         <v>6</v>
@@ -1381,20 +1362,20 @@
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A23">
-        <v>20</v>
+        <v>100</v>
       </c>
       <c r="B23" t="s">
-        <v>131</v>
+        <v>99</v>
       </c>
       <c r="C23" t="str">
         <f t="shared" si="0"/>
-        <v>MZB0NBWEU</v>
+        <v>MZB0JRIEU</v>
       </c>
       <c r="D23" s="3">
-        <v>6932554496944</v>
+        <v>6932554425814</v>
       </c>
       <c r="E23">
-        <v>363</v>
+        <v>67</v>
       </c>
       <c r="F23" t="s">
         <v>6</v>
@@ -1402,20 +1383,20 @@
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A24">
-        <v>80</v>
+        <v>40</v>
       </c>
       <c r="B24" t="s">
-        <v>118</v>
+        <v>100</v>
       </c>
       <c r="C24" t="str">
         <f t="shared" si="0"/>
-        <v>MZB0JSEEU</v>
+        <v>MZB0JSAEU</v>
       </c>
       <c r="D24" s="3">
-        <v>6932554425104</v>
+        <v>6932554424978</v>
       </c>
       <c r="E24">
-        <v>68</v>
+        <v>79</v>
       </c>
       <c r="F24" t="s">
         <v>6</v>
@@ -1423,20 +1404,20 @@
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="B25" t="s">
-        <v>119</v>
+        <v>101</v>
       </c>
       <c r="C25" t="str">
         <f t="shared" si="0"/>
-        <v>MZB0JTEEU</v>
+        <v>MZB0JSTEU</v>
       </c>
       <c r="D25" s="3">
-        <v>6932554425432</v>
+        <v>6932554425241</v>
       </c>
       <c r="E25">
-        <v>68</v>
+        <v>79</v>
       </c>
       <c r="F25" t="s">
         <v>6</v>
@@ -1444,20 +1425,20 @@
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26">
-        <v>100</v>
+        <v>40</v>
       </c>
       <c r="B26" t="s">
-        <v>120</v>
+        <v>102</v>
       </c>
       <c r="C26" t="str">
         <f t="shared" si="0"/>
-        <v>MZB0JRIEU</v>
+        <v>MZB0JTPEU</v>
       </c>
       <c r="D26" s="3">
-        <v>6932554425814</v>
+        <v>6932554425548</v>
       </c>
       <c r="E26">
-        <v>68</v>
+        <v>79</v>
       </c>
       <c r="F26" t="s">
         <v>6</v>
@@ -1465,20 +1446,20 @@
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27">
-        <v>100</v>
+        <v>5</v>
       </c>
       <c r="B27" t="s">
-        <v>121</v>
+        <v>103</v>
       </c>
       <c r="C27" t="str">
         <f t="shared" si="0"/>
-        <v>MZB0JSAEU</v>
+        <v>MZB0N5WEU</v>
       </c>
       <c r="D27" s="3">
-        <v>6932554424978</v>
+        <v>6932554493295</v>
       </c>
       <c r="E27">
-        <v>87</v>
+        <v>79</v>
       </c>
       <c r="F27" t="s">
         <v>6</v>
@@ -1486,20 +1467,20 @@
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28">
-        <v>100</v>
+        <v>5</v>
       </c>
       <c r="B28" t="s">
-        <v>122</v>
+        <v>104</v>
       </c>
       <c r="C28" t="str">
         <f t="shared" si="0"/>
-        <v>MZB0JSTEU</v>
+        <v>MZB0N5TEU</v>
       </c>
       <c r="D28" s="3">
-        <v>6932554425241</v>
+        <v>6932554493264</v>
       </c>
       <c r="E28">
-        <v>87</v>
+        <v>79</v>
       </c>
       <c r="F28" t="s">
         <v>6</v>
@@ -1507,20 +1488,20 @@
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29">
-        <v>100</v>
+        <v>5</v>
       </c>
       <c r="B29" t="s">
-        <v>123</v>
+        <v>105</v>
       </c>
       <c r="C29" t="str">
         <f t="shared" si="0"/>
-        <v>MZB0JTPEU</v>
+        <v>MZB0N5QEU</v>
       </c>
       <c r="D29" s="3">
-        <v>6932554425548</v>
+        <v>6932554493257</v>
       </c>
       <c r="E29">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="F29" t="s">
         <v>6</v>
@@ -1528,20 +1509,20 @@
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="B30" t="s">
-        <v>124</v>
+        <v>61</v>
       </c>
       <c r="C30" t="str">
         <f t="shared" si="0"/>
-        <v>MZB0N5WEU</v>
+        <v>MZB0KTPEU</v>
       </c>
       <c r="D30" s="3">
-        <v>6932554493295</v>
+        <v>6932554447144</v>
       </c>
       <c r="E30">
-        <v>89</v>
+        <v>100</v>
       </c>
       <c r="F30" t="s">
         <v>6</v>
@@ -1552,17 +1533,17 @@
         <v>5</v>
       </c>
       <c r="B31" t="s">
-        <v>125</v>
+        <v>62</v>
       </c>
       <c r="C31" t="str">
         <f t="shared" si="0"/>
-        <v>MZB0N5TEU</v>
+        <v>MZB0LBMEU</v>
       </c>
       <c r="D31" s="3">
-        <v>6932554493264</v>
+        <v>6932554455927</v>
       </c>
       <c r="E31">
-        <v>89</v>
+        <v>100</v>
       </c>
       <c r="F31" t="s">
         <v>6</v>
@@ -1570,20 +1551,20 @@
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="B32" t="s">
-        <v>126</v>
+        <v>63</v>
       </c>
       <c r="C32" t="str">
         <f t="shared" si="0"/>
-        <v>MZB0N5QEU</v>
+        <v>MZB0LBVEU</v>
       </c>
       <c r="D32" s="3">
-        <v>6932554493257</v>
+        <v>6932554455934</v>
       </c>
       <c r="E32">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="F32" t="s">
         <v>6</v>
@@ -1591,20 +1572,20 @@
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="B33" t="s">
-        <v>73</v>
+        <v>21</v>
       </c>
       <c r="C33" t="str">
         <f t="shared" si="0"/>
-        <v>MZB0KTPEU</v>
+        <v>MZB0M8FEU</v>
       </c>
       <c r="D33" s="3">
-        <v>6932554447144</v>
+        <v>6932554476274</v>
       </c>
       <c r="E33">
-        <v>102</v>
+        <v>135</v>
       </c>
       <c r="F33" t="s">
         <v>6</v>
@@ -1612,20 +1593,20 @@
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="B34" t="s">
-        <v>74</v>
+        <v>106</v>
       </c>
       <c r="C34" t="str">
         <f t="shared" si="0"/>
-        <v>MZB0LBMEU</v>
+        <v>MZB0LWMEU</v>
       </c>
       <c r="D34" s="3">
-        <v>6932554455927</v>
+        <v>6932554469252</v>
       </c>
       <c r="E34">
-        <v>102</v>
+        <v>175</v>
       </c>
       <c r="F34" t="s">
         <v>6</v>
@@ -1633,20 +1614,20 @@
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="B35" t="s">
-        <v>75</v>
+        <v>22</v>
       </c>
       <c r="C35" t="str">
         <f t="shared" si="0"/>
-        <v>MZB0LBVEU</v>
+        <v>VHU6253EU</v>
       </c>
       <c r="D35" s="3">
-        <v>6932554455934</v>
+        <v>6932554467319</v>
       </c>
       <c r="E35">
-        <v>102</v>
+        <v>165</v>
       </c>
       <c r="F35" t="s">
         <v>6</v>
@@ -1654,20 +1635,20 @@
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="B36" t="s">
-        <v>25</v>
+        <v>125</v>
       </c>
       <c r="C36" t="str">
         <f t="shared" si="0"/>
-        <v>MZB0M8FEU</v>
+        <v>VHU6302EU</v>
       </c>
       <c r="D36" s="3">
-        <v>6932554476274</v>
+        <v>6932554467937</v>
       </c>
       <c r="E36">
-        <v>143</v>
+        <v>185</v>
       </c>
       <c r="F36" t="s">
         <v>6</v>
@@ -1675,20 +1656,20 @@
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37">
-        <v>5</v>
+        <v>100</v>
       </c>
       <c r="B37" t="s">
-        <v>26</v>
+        <v>108</v>
       </c>
       <c r="C37" t="str">
         <f t="shared" si="0"/>
-        <v>MZB0MOIEU</v>
+        <v>C338E</v>
       </c>
       <c r="D37" s="3">
-        <v>6932554482688</v>
+        <v>3030050069419</v>
       </c>
       <c r="E37">
-        <v>143</v>
+        <v>19</v>
       </c>
       <c r="F37" t="s">
         <v>6</v>
@@ -1696,20 +1677,20 @@
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="B38" t="s">
-        <v>127</v>
+        <v>109</v>
       </c>
       <c r="C38" t="str">
         <f t="shared" si="0"/>
-        <v>MZB0LWMEU</v>
+        <v>AS962E</v>
       </c>
       <c r="D38" s="3">
-        <v>6932554469252</v>
+        <v>3030050182637</v>
       </c>
       <c r="E38">
-        <v>179</v>
+        <v>37</v>
       </c>
       <c r="F38" t="s">
         <v>6</v>
@@ -1717,20 +1698,20 @@
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39">
-        <v>10</v>
+        <v>45</v>
       </c>
       <c r="B39" t="s">
-        <v>128</v>
+        <v>110</v>
       </c>
       <c r="C39" t="str">
         <f t="shared" si="0"/>
-        <v>MZB0LWKEU</v>
+        <v>AS960E</v>
       </c>
       <c r="D39" s="3">
-        <v>6932554469221</v>
+        <v>3030050165357</v>
       </c>
       <c r="E39">
-        <v>179</v>
+        <v>41</v>
       </c>
       <c r="F39" t="s">
         <v>6</v>
@@ -1738,20 +1719,20 @@
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40">
-        <v>5</v>
+        <v>136</v>
       </c>
       <c r="B40" t="s">
-        <v>60</v>
+        <v>123</v>
       </c>
       <c r="C40" t="str">
         <f t="shared" si="0"/>
-        <v>MZB0LYMEU</v>
+        <v>TAT6A513</v>
       </c>
       <c r="D40" s="3">
-        <v>6932554469825</v>
+        <v>4242005369782</v>
       </c>
       <c r="E40">
-        <v>179</v>
+        <v>20.680000000000003</v>
       </c>
       <c r="F40" t="s">
         <v>6</v>
@@ -1759,86 +1740,86 @@
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="B41" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="C41" t="str">
         <f t="shared" si="0"/>
-        <v>MZB0MI3EU</v>
+        <v>27F650R</v>
       </c>
       <c r="D41" s="3">
-        <v>6932554495701</v>
+        <v>8592344400261</v>
       </c>
       <c r="E41">
-        <v>267</v>
+        <v>95</v>
       </c>
       <c r="F41" t="s">
-        <v>6</v>
+        <v>145</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42">
-        <v>5</v>
+        <v>105</v>
       </c>
       <c r="B42" t="s">
-        <v>72</v>
+        <v>81</v>
       </c>
       <c r="C42" t="str">
         <f t="shared" si="0"/>
-        <v>MZB0MIGEU</v>
+        <v>CAF-TF101S-AEUR</v>
       </c>
       <c r="D42" s="3">
-        <v>6932554481995</v>
+        <v>810123673285</v>
       </c>
       <c r="E42">
-        <v>267</v>
+        <v>135</v>
       </c>
       <c r="F42" t="s">
-        <v>6</v>
+        <v>145</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43">
-        <v>5</v>
+        <v>35</v>
       </c>
       <c r="B43" t="s">
-        <v>27</v>
+        <v>82</v>
       </c>
       <c r="C43" t="str">
         <f t="shared" si="0"/>
-        <v>VHU6253EU</v>
+        <v>CAF-DC121-ADER</v>
       </c>
       <c r="D43" s="3">
-        <v>6932554467319</v>
+        <v>810123675227</v>
       </c>
       <c r="E43">
-        <v>165</v>
+        <v>123</v>
       </c>
       <c r="F43" t="s">
-        <v>6</v>
+        <v>145</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44">
-        <v>5</v>
+        <v>30</v>
       </c>
       <c r="B44" t="s">
-        <v>158</v>
+        <v>55</v>
       </c>
       <c r="C44" t="str">
         <f t="shared" si="0"/>
-        <v>VHU6302EU</v>
+        <v>486236-01</v>
       </c>
       <c r="D44" s="3">
-        <v>6932554467937</v>
+        <v>5025155096772</v>
       </c>
       <c r="E44">
-        <v>185</v>
+        <v>309</v>
       </c>
       <c r="F44" t="s">
-        <v>160</v>
+        <v>145</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.25">
@@ -1846,20 +1827,20 @@
         <v>10</v>
       </c>
       <c r="B45" t="s">
-        <v>20</v>
+        <v>56</v>
       </c>
       <c r="C45" t="str">
         <f t="shared" si="0"/>
-        <v>B11W6AT</v>
+        <v>492963-01</v>
       </c>
       <c r="D45" s="3">
-        <v>198828212467</v>
+        <v>5025155114834</v>
       </c>
       <c r="E45">
-        <v>110</v>
+        <v>565</v>
       </c>
       <c r="F45" t="s">
-        <v>7</v>
+        <v>145</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.25">
@@ -1867,17 +1848,17 @@
         <v>100</v>
       </c>
       <c r="B46" t="s">
-        <v>134</v>
+        <v>128</v>
       </c>
       <c r="C46" t="str">
         <f t="shared" si="0"/>
-        <v>C338E</v>
+        <v>W-SO01-0004</v>
       </c>
       <c r="D46" s="3">
-        <v>3030050069419</v>
+        <v>6970135030484</v>
       </c>
       <c r="E46">
-        <v>19</v>
+        <v>6</v>
       </c>
       <c r="F46" t="s">
         <v>6</v>
@@ -1885,23 +1866,23 @@
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A47">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="B47" t="s">
-        <v>135</v>
+        <v>129</v>
       </c>
       <c r="C47" t="str">
         <f t="shared" si="0"/>
-        <v>C451E</v>
+        <v>WG851-11EDR</v>
       </c>
       <c r="D47" s="3">
-        <v>3030050153644</v>
+        <v>6970135033836</v>
       </c>
       <c r="E47">
-        <v>21</v>
+        <v>309</v>
       </c>
       <c r="F47" t="s">
-        <v>6</v>
+        <v>145</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.25">
@@ -1909,59 +1890,59 @@
         <v>10</v>
       </c>
       <c r="B48" t="s">
-        <v>159</v>
+        <v>130</v>
       </c>
       <c r="C48" t="str">
         <f t="shared" si="0"/>
-        <v>E976E</v>
+        <v>WG852-11EDR</v>
       </c>
       <c r="D48" s="3">
-        <v>3030050153231</v>
+        <v>6970135035403</v>
       </c>
       <c r="E48">
-        <v>28</v>
+        <v>239</v>
       </c>
       <c r="F48" t="s">
-        <v>6</v>
+        <v>145</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A49">
-        <v>40</v>
+        <v>10</v>
       </c>
       <c r="B49" t="s">
-        <v>136</v>
+        <v>16</v>
       </c>
       <c r="C49" t="str">
         <f t="shared" si="0"/>
-        <v>AS962E</v>
+        <v>B11W6AT</v>
       </c>
       <c r="D49" s="3">
-        <v>3030050182637</v>
+        <v>198828212467</v>
       </c>
       <c r="E49">
-        <v>37</v>
+        <v>110</v>
       </c>
       <c r="F49" t="s">
-        <v>6</v>
+        <v>145</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="B50" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="C50" t="str">
         <f t="shared" si="0"/>
-        <v>AS960E</v>
+        <v>55020EYL</v>
       </c>
       <c r="D50" s="3">
-        <v>3030050165357</v>
+        <v>6942103155024</v>
       </c>
       <c r="E50">
-        <v>41</v>
+        <v>89</v>
       </c>
       <c r="F50" t="s">
         <v>6</v>
@@ -1969,220 +1950,220 @@
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51">
-        <v>136</v>
+        <v>25</v>
       </c>
       <c r="B51" t="s">
-        <v>155</v>
+        <v>132</v>
       </c>
       <c r="C51" t="str">
         <f t="shared" si="0"/>
-        <v>TAT6A513</v>
+        <v>55020DKM</v>
       </c>
       <c r="D51" s="3">
-        <v>4242005369782</v>
+        <v>6942103132001</v>
       </c>
       <c r="E51">
-        <v>20.680000000000003</v>
+        <v>105</v>
       </c>
       <c r="F51" t="s">
-        <v>161</v>
+        <v>6</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52">
-        <v>150</v>
+        <v>5</v>
       </c>
       <c r="B52" t="s">
-        <v>97</v>
+        <v>133</v>
       </c>
       <c r="C52" t="str">
         <f t="shared" si="0"/>
-        <v>CAF-TF101S-AEUR</v>
+        <v>55020DJT</v>
       </c>
       <c r="D52" s="3">
-        <v>810123673285</v>
+        <v>6942103131967</v>
       </c>
       <c r="E52">
-        <v>135</v>
+        <v>119</v>
       </c>
       <c r="F52" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53">
-        <v>40</v>
+        <v>5</v>
       </c>
       <c r="B53" t="s">
-        <v>98</v>
+        <v>134</v>
       </c>
       <c r="C53" t="str">
         <f t="shared" si="0"/>
-        <v>CAF-DC121-ADER</v>
+        <v>55020DKH</v>
       </c>
       <c r="D53" s="3">
-        <v>810123675227</v>
+        <v>6942103132025</v>
       </c>
       <c r="E53">
-        <v>123</v>
+        <v>119</v>
       </c>
       <c r="F53" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="B54" t="s">
-        <v>65</v>
+        <v>135</v>
       </c>
       <c r="C54" t="str">
         <f t="shared" si="0"/>
-        <v>486236-01</v>
+        <v>55020DJQ</v>
       </c>
       <c r="D54" s="3">
-        <v>5025155096772</v>
+        <v>6942103131981</v>
       </c>
       <c r="E54">
-        <v>309</v>
+        <v>144</v>
       </c>
       <c r="F54" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="B55" t="s">
-        <v>66</v>
+        <v>136</v>
       </c>
       <c r="C55" t="str">
         <f t="shared" si="0"/>
-        <v>492963-01</v>
+        <v>55020DKD</v>
       </c>
       <c r="D55" s="3">
-        <v>5025155114834</v>
+        <v>6942103132032</v>
       </c>
       <c r="E55">
-        <v>565</v>
+        <v>155</v>
       </c>
       <c r="F55" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A56">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="B56" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C56" t="str">
         <f t="shared" si="0"/>
-        <v>JBLPBENCORE2EP</v>
+        <v>55020EWB</v>
       </c>
       <c r="D56" s="3">
-        <v>1200130020216</v>
+        <v>6942103154300</v>
       </c>
       <c r="E56">
-        <v>185</v>
+        <v>209</v>
       </c>
       <c r="F56" t="s">
-        <v>161</v>
+        <v>6</v>
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A57">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="B57" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C57" t="str">
         <f t="shared" si="0"/>
-        <v>JBLPBENCOREESS2EP</v>
+        <v>55020FTP</v>
       </c>
       <c r="D57" s="3">
-        <v>1200130022517</v>
+        <v>6942103168239</v>
       </c>
       <c r="E57">
-        <v>132</v>
+        <v>189</v>
       </c>
       <c r="F57" t="s">
-        <v>161</v>
+        <v>6</v>
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A58">
-        <v>40</v>
+        <v>5</v>
       </c>
       <c r="B58" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C58" t="str">
         <f t="shared" si="0"/>
-        <v>JBLT530BTBEGEU</v>
+        <v>55020FTT</v>
       </c>
       <c r="D58" s="3">
-        <v>1200130029998</v>
+        <v>6942103168192</v>
       </c>
       <c r="E58">
-        <v>29</v>
+        <v>311</v>
       </c>
       <c r="F58" t="s">
-        <v>161</v>
+        <v>6</v>
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A59">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="B59" t="s">
-        <v>141</v>
+        <v>111</v>
       </c>
       <c r="C59" t="str">
         <f t="shared" si="0"/>
-        <v>JBLT530BTBLKEU</v>
+        <v>JBLPBENCORE2EP</v>
       </c>
       <c r="D59" s="3">
-        <v>1200130029967</v>
+        <v>1200130020216</v>
       </c>
       <c r="E59">
-        <v>29</v>
+        <v>185</v>
       </c>
       <c r="F59" t="s">
-        <v>161</v>
+        <v>6</v>
       </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A60">
-        <v>70</v>
+        <v>50</v>
       </c>
       <c r="B60" t="s">
-        <v>142</v>
+        <v>112</v>
       </c>
       <c r="C60" t="str">
         <f t="shared" si="0"/>
-        <v>JBLT530BTLAVEU</v>
+        <v>JBLPBENCOREESS2EP</v>
       </c>
       <c r="D60" s="3">
-        <v>1200130030000</v>
+        <v>1200130022517</v>
       </c>
       <c r="E60">
-        <v>29</v>
+        <v>132</v>
       </c>
       <c r="F60" t="s">
-        <v>161</v>
+        <v>6</v>
       </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A61">
-        <v>130</v>
+        <v>60</v>
       </c>
       <c r="B61" t="s">
-        <v>116</v>
+        <v>97</v>
       </c>
       <c r="C61" t="str">
         <f t="shared" si="0"/>
@@ -2195,18 +2176,18 @@
         <v>40</v>
       </c>
       <c r="F61" t="s">
-        <v>7</v>
+        <v>145</v>
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A62">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="B62" t="s">
-        <v>59</v>
+        <v>51</v>
       </c>
       <c r="C62" t="str">
-        <f t="shared" si="0"/>
+        <f t="shared" ref="C62:C125" si="1">MID(B62,FIND("@",SUBSTITUTE(B62," ","@",LEN(B62)-LEN(SUBSTITUTE(B62," ",""))))+1,LEN(B62))</f>
         <v>1.633-701.0</v>
       </c>
       <c r="D62" s="3">
@@ -2216,7 +2197,7 @@
         <v>49</v>
       </c>
       <c r="F62" t="s">
-        <v>7</v>
+        <v>145</v>
       </c>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.25">
@@ -2224,10 +2205,10 @@
         <v>5</v>
       </c>
       <c r="B63" t="s">
-        <v>57</v>
+        <v>49</v>
       </c>
       <c r="C63" t="str">
-        <f t="shared" ref="C63:C126" si="1">MID(B63,FIND("@",SUBSTITUTE(B63," ","@",LEN(B63)-LEN(SUBSTITUTE(B63," ",""))))+1,LEN(B63))</f>
+        <f t="shared" si="1"/>
         <v>1.633-514.0</v>
       </c>
       <c r="D63" s="3">
@@ -2237,7 +2218,7 @@
         <v>61</v>
       </c>
       <c r="F63" t="s">
-        <v>7</v>
+        <v>145</v>
       </c>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.25">
@@ -2245,7 +2226,7 @@
         <v>10</v>
       </c>
       <c r="B64" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
       <c r="C64" t="str">
         <f t="shared" si="1"/>
@@ -2258,15 +2239,15 @@
         <v>99</v>
       </c>
       <c r="F64" t="s">
-        <v>7</v>
+        <v>145</v>
       </c>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="B65" t="s">
-        <v>113</v>
+        <v>94</v>
       </c>
       <c r="C65" t="str">
         <f t="shared" si="1"/>
@@ -2279,7 +2260,7 @@
         <v>114</v>
       </c>
       <c r="F65" t="s">
-        <v>7</v>
+        <v>145</v>
       </c>
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.25">
@@ -2287,7 +2268,7 @@
         <v>20</v>
       </c>
       <c r="B66" t="s">
-        <v>114</v>
+        <v>95</v>
       </c>
       <c r="C66" t="str">
         <f t="shared" si="1"/>
@@ -2300,7 +2281,7 @@
         <v>157</v>
       </c>
       <c r="F66" t="s">
-        <v>7</v>
+        <v>145</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
@@ -2308,7 +2289,7 @@
         <v>10</v>
       </c>
       <c r="B67" t="s">
-        <v>143</v>
+        <v>113</v>
       </c>
       <c r="C67" t="str">
         <f t="shared" si="1"/>
@@ -2321,7 +2302,7 @@
         <v>72.600000000000009</v>
       </c>
       <c r="F67" t="s">
-        <v>161</v>
+        <v>145</v>
       </c>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.25">
@@ -2329,7 +2310,7 @@
         <v>40</v>
       </c>
       <c r="B68" t="s">
-        <v>77</v>
+        <v>64</v>
       </c>
       <c r="C68" t="str">
         <f t="shared" si="1"/>
@@ -2347,10 +2328,10 @@
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A69">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="B69" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="C69" t="str">
         <f t="shared" si="1"/>
@@ -2371,7 +2352,7 @@
         <v>30</v>
       </c>
       <c r="B70" t="s">
-        <v>61</v>
+        <v>52</v>
       </c>
       <c r="C70" t="str">
         <f t="shared" si="1"/>
@@ -2392,7 +2373,7 @@
         <v>45</v>
       </c>
       <c r="B71" t="s">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="C71" t="str">
         <f t="shared" si="1"/>
@@ -2405,15 +2386,15 @@
         <v>29</v>
       </c>
       <c r="F71" t="s">
-        <v>7</v>
+        <v>145</v>
       </c>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A72">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="B72" t="s">
-        <v>78</v>
+        <v>65</v>
       </c>
       <c r="C72" t="str">
         <f t="shared" si="1"/>
@@ -2426,15 +2407,15 @@
         <v>121</v>
       </c>
       <c r="F72" t="s">
-        <v>7</v>
+        <v>145</v>
       </c>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A73">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="B73" t="s">
-        <v>79</v>
+        <v>66</v>
       </c>
       <c r="C73" t="str">
         <f t="shared" si="1"/>
@@ -2447,7 +2428,7 @@
         <v>130</v>
       </c>
       <c r="F73" t="s">
-        <v>7</v>
+        <v>145</v>
       </c>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.25">
@@ -2455,7 +2436,7 @@
         <v>60</v>
       </c>
       <c r="B74" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C74" t="str">
         <f t="shared" si="1"/>
@@ -2468,15 +2449,15 @@
         <v>145</v>
       </c>
       <c r="F74" t="s">
-        <v>7</v>
+        <v>145</v>
       </c>
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A75">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="B75" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="C75" t="str">
         <f t="shared" si="1"/>
@@ -2489,15 +2470,15 @@
         <v>147</v>
       </c>
       <c r="F75" t="s">
-        <v>7</v>
+        <v>145</v>
       </c>
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A76">
+        <v>10</v>
+      </c>
+      <c r="B76" t="s">
         <v>15</v>
-      </c>
-      <c r="B76" t="s">
-        <v>19</v>
       </c>
       <c r="C76" t="str">
         <f t="shared" si="1"/>
@@ -2510,15 +2491,15 @@
         <v>112</v>
       </c>
       <c r="F76" t="s">
-        <v>7</v>
+        <v>145</v>
       </c>
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A77">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="B77" t="s">
-        <v>67</v>
+        <v>57</v>
       </c>
       <c r="C77" t="str">
         <f t="shared" si="1"/>
@@ -2531,7 +2512,7 @@
         <v>157</v>
       </c>
       <c r="F77" t="s">
-        <v>7</v>
+        <v>145</v>
       </c>
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.25">
@@ -2539,62 +2520,62 @@
         <v>5</v>
       </c>
       <c r="B78" t="s">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="C78" t="str">
         <f t="shared" si="1"/>
-        <v>ES501EU</v>
+        <v>ES701EU</v>
       </c>
       <c r="D78" s="3">
-        <v>622356301824</v>
+        <v>622356289825</v>
       </c>
       <c r="E78">
-        <v>252</v>
+        <v>410</v>
       </c>
       <c r="F78" t="s">
-        <v>7</v>
+        <v>145</v>
       </c>
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A79">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="B79" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C79" t="str">
         <f t="shared" si="1"/>
-        <v>ES701EU</v>
+        <v>CB100EU</v>
       </c>
       <c r="D79" s="3">
-        <v>622356289825</v>
+        <v>622356236775</v>
       </c>
       <c r="E79">
-        <v>410</v>
+        <v>85</v>
       </c>
       <c r="F79" t="s">
-        <v>7</v>
+        <v>145</v>
       </c>
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A80">
-        <v>15</v>
+        <v>200</v>
       </c>
       <c r="B80" t="s">
-        <v>29</v>
+        <v>114</v>
       </c>
       <c r="C80" t="str">
         <f t="shared" si="1"/>
-        <v>CB100EU</v>
+        <v>426967</v>
       </c>
       <c r="D80" s="3">
-        <v>622356236775</v>
+        <v>4210201426967</v>
       </c>
       <c r="E80">
-        <v>85</v>
+        <v>15.400000000000002</v>
       </c>
       <c r="F80" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.25">
@@ -2602,214 +2583,214 @@
         <v>200</v>
       </c>
       <c r="B81" t="s">
-        <v>144</v>
+        <v>115</v>
       </c>
       <c r="C81" t="str">
         <f t="shared" si="1"/>
-        <v>426967</v>
+        <v>446392</v>
       </c>
       <c r="D81" s="3">
-        <v>4210201426967</v>
+        <v>4210201446392</v>
       </c>
       <c r="E81">
         <v>15.400000000000002</v>
       </c>
       <c r="F81" t="s">
-        <v>161</v>
+        <v>6</v>
       </c>
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A82">
-        <v>200</v>
+        <v>120</v>
       </c>
       <c r="B82" t="s">
-        <v>145</v>
+        <v>116</v>
       </c>
       <c r="C82" t="str">
         <f t="shared" si="1"/>
-        <v>446392</v>
+        <v>D103</v>
       </c>
       <c r="D82" s="3">
-        <v>4210201446392</v>
+        <v>4210201432227</v>
       </c>
       <c r="E82">
-        <v>15.400000000000002</v>
+        <v>29.150000000000002</v>
       </c>
       <c r="F82" t="s">
-        <v>161</v>
+        <v>6</v>
       </c>
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A83">
-        <v>126</v>
+        <v>50</v>
       </c>
       <c r="B83" t="s">
-        <v>146</v>
+        <v>117</v>
       </c>
       <c r="C83" t="str">
         <f t="shared" si="1"/>
-        <v>D103</v>
+        <v>914170</v>
       </c>
       <c r="D83" s="3">
-        <v>4210201432227</v>
+        <v>8001090914415</v>
       </c>
       <c r="E83">
-        <v>29.150000000000002</v>
+        <v>24.750000000000004</v>
       </c>
       <c r="F83" t="s">
-        <v>161</v>
+        <v>6</v>
       </c>
     </row>
     <row r="84" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A84">
-        <v>50</v>
+        <v>80</v>
       </c>
       <c r="B84" t="s">
-        <v>147</v>
+        <v>118</v>
       </c>
       <c r="C84" t="str">
         <f t="shared" si="1"/>
-        <v>914170</v>
+        <v>3216721</v>
       </c>
       <c r="D84" s="3">
-        <v>8001090914415</v>
+        <v>8001090914941</v>
       </c>
       <c r="E84">
         <v>24.750000000000004</v>
       </c>
       <c r="F84" t="s">
-        <v>161</v>
+        <v>6</v>
       </c>
     </row>
     <row r="85" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A85">
-        <v>80</v>
+        <v>110</v>
       </c>
       <c r="B85" t="s">
-        <v>148</v>
-      </c>
-      <c r="C85" t="str">
-        <f t="shared" si="1"/>
-        <v>3216721</v>
+        <v>119</v>
+      </c>
+      <c r="C85" s="5" t="s">
+        <v>18</v>
       </c>
       <c r="D85" s="3">
-        <v>8001090914941</v>
+        <v>8006530069373</v>
       </c>
       <c r="E85">
-        <v>24.750000000000004</v>
+        <v>58.300000000000004</v>
       </c>
       <c r="F85" t="s">
-        <v>161</v>
+        <v>6</v>
       </c>
     </row>
     <row r="86" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A86">
-        <v>117</v>
+        <v>140</v>
       </c>
       <c r="B86" t="s">
-        <v>149</v>
+        <v>120</v>
       </c>
       <c r="C86" s="5" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="D86" s="3">
-        <v>8006530069373</v>
+        <v>8006540773307</v>
       </c>
       <c r="E86">
-        <v>58.300000000000004</v>
+        <v>17.380000000000003</v>
       </c>
       <c r="F86" t="s">
-        <v>161</v>
+        <v>6</v>
       </c>
     </row>
     <row r="87" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A87">
-        <v>144</v>
+        <v>138</v>
       </c>
       <c r="B87" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="C87" s="5" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="D87" s="3">
-        <v>8006540773307</v>
+        <v>8700216297172</v>
       </c>
       <c r="E87">
         <v>17.380000000000003</v>
       </c>
       <c r="F87" t="s">
-        <v>161</v>
+        <v>6</v>
       </c>
     </row>
     <row r="88" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A88">
-        <v>138</v>
+        <v>200</v>
       </c>
       <c r="B88" t="s">
-        <v>151</v>
-      </c>
-      <c r="C88" s="5" t="s">
-        <v>22</v>
+        <v>53</v>
+      </c>
+      <c r="C88" t="str">
+        <f t="shared" si="1"/>
+        <v>NA352/00</v>
       </c>
       <c r="D88" s="3">
-        <v>8700216297172</v>
+        <v>8720389032998</v>
       </c>
       <c r="E88">
-        <v>17.380000000000003</v>
+        <v>93</v>
       </c>
       <c r="F88" t="s">
-        <v>161</v>
+        <v>145</v>
       </c>
     </row>
     <row r="89" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A89">
-        <v>200</v>
+        <v>50</v>
       </c>
       <c r="B89" t="s">
-        <v>62</v>
+        <v>10</v>
       </c>
       <c r="C89" t="str">
         <f t="shared" si="1"/>
-        <v>NA352/00</v>
+        <v>BRI940/00</v>
       </c>
       <c r="D89" s="3">
-        <v>8720389032998</v>
+        <v>8720689020206</v>
       </c>
       <c r="E89">
-        <v>93</v>
+        <v>199</v>
       </c>
       <c r="F89" t="s">
-        <v>7</v>
+        <v>145</v>
       </c>
     </row>
     <row r="90" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A90">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="B90" t="s">
-        <v>11</v>
+        <v>124</v>
       </c>
       <c r="C90" t="str">
         <f t="shared" si="1"/>
-        <v>BRI940/00</v>
+        <v>BHD302/10</v>
       </c>
       <c r="D90" s="3">
-        <v>8720689020206</v>
+        <v>8710103959533</v>
       </c>
       <c r="E90">
-        <v>199</v>
+        <v>10</v>
       </c>
       <c r="F90" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="91" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A91">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="B91" t="s">
-        <v>115</v>
+        <v>96</v>
       </c>
       <c r="C91" t="str">
         <f t="shared" si="1"/>
@@ -2822,45 +2803,44 @@
         <v>280</v>
       </c>
       <c r="F91" t="s">
-        <v>7</v>
+        <v>145</v>
       </c>
     </row>
     <row r="92" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A92">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="B92" t="s">
-        <v>156</v>
-      </c>
-      <c r="C92" t="str">
-        <f t="shared" si="1"/>
-        <v>BHD302/10</v>
+        <v>42</v>
+      </c>
+      <c r="C92" s="5" t="s">
+        <v>18</v>
       </c>
       <c r="D92" s="3">
-        <v>8710103959533</v>
+        <v>6941764428546</v>
       </c>
       <c r="E92">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F92" t="s">
-        <v>161</v>
+        <v>6</v>
       </c>
     </row>
     <row r="93" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A93">
-        <v>150</v>
+        <v>80</v>
       </c>
       <c r="B93" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="C93" s="5" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="D93" s="3">
-        <v>6941764428546</v>
+        <v>6941764467194</v>
       </c>
       <c r="E93">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="F93" t="s">
         <v>6</v>
@@ -2868,19 +2848,19 @@
     </row>
     <row r="94" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A94">
-        <v>90</v>
+        <v>120</v>
       </c>
       <c r="B94" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="C94" s="5" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="D94" s="3">
-        <v>6941764467194</v>
+        <v>6941764432994</v>
       </c>
       <c r="E94">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="F94" t="s">
         <v>6</v>
@@ -2888,19 +2868,19 @@
     </row>
     <row r="95" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A95">
-        <v>120</v>
+        <v>10</v>
       </c>
       <c r="B95" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="C95" s="5" t="s">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="D95" s="3">
-        <v>6941764432994</v>
+        <v>6941764483408</v>
       </c>
       <c r="E95">
-        <v>19</v>
+        <v>39</v>
       </c>
       <c r="F95" t="s">
         <v>6</v>
@@ -2908,19 +2888,20 @@
     </row>
     <row r="96" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A96">
-        <v>15</v>
+        <v>40</v>
       </c>
       <c r="B96" t="s">
-        <v>52</v>
-      </c>
-      <c r="C96" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="C96" t="str">
+        <f t="shared" si="1"/>
+        <v>MB4700</v>
+      </c>
+      <c r="D96" s="3">
+        <v>4008496942060</v>
+      </c>
+      <c r="E96">
         <v>22</v>
-      </c>
-      <c r="D96" s="3">
-        <v>6941764483408</v>
-      </c>
-      <c r="E96">
-        <v>39</v>
       </c>
       <c r="F96" t="s">
         <v>6</v>
@@ -2928,41 +2909,41 @@
     </row>
     <row r="97" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A97">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="B97" t="s">
-        <v>13</v>
+        <v>121</v>
       </c>
       <c r="C97" t="str">
         <f t="shared" si="1"/>
-        <v>S9300</v>
+        <v>26510-56</v>
       </c>
       <c r="D97" s="3">
-        <v>5038061105520</v>
+        <v>5038061142860</v>
       </c>
       <c r="E97">
-        <v>31</v>
+        <v>38.5</v>
       </c>
       <c r="F97" t="s">
-        <v>6</v>
+        <v>145</v>
       </c>
     </row>
     <row r="98" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A98">
-        <v>40</v>
+        <v>1600</v>
       </c>
       <c r="B98" t="s">
-        <v>37</v>
+        <v>140</v>
       </c>
       <c r="C98" t="str">
         <f t="shared" si="1"/>
-        <v>MB4700</v>
+        <v>EI-T5600BBEGEU</v>
       </c>
       <c r="D98" s="3">
-        <v>4008496942060</v>
+        <v>8806095039893</v>
       </c>
       <c r="E98">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="F98" t="s">
         <v>6</v>
@@ -2970,41 +2951,41 @@
     </row>
     <row r="99" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A99">
-        <v>33</v>
+        <v>850</v>
       </c>
       <c r="B99" t="s">
-        <v>152</v>
+        <v>141</v>
       </c>
       <c r="C99" t="str">
         <f t="shared" si="1"/>
-        <v>26510-56</v>
+        <v>EI-T5600BWEGEU</v>
       </c>
       <c r="D99" s="3">
-        <v>5038061142860</v>
+        <v>8806095039824</v>
       </c>
       <c r="E99">
-        <v>38.5</v>
+        <v>12</v>
       </c>
       <c r="F99" t="s">
-        <v>161</v>
+        <v>6</v>
       </c>
     </row>
     <row r="100" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A100">
-        <v>60</v>
+        <v>450</v>
       </c>
       <c r="B100" t="s">
-        <v>14</v>
+        <v>142</v>
       </c>
       <c r="C100" t="str">
         <f t="shared" si="1"/>
-        <v>EB-P3400XUEGEU</v>
+        <v>SM-R390NZAAMEA</v>
       </c>
       <c r="D100" s="3">
-        <v>8806094682748</v>
+        <v>8806095380384</v>
       </c>
       <c r="E100">
-        <v>16</v>
+        <v>29</v>
       </c>
       <c r="F100" t="s">
         <v>6</v>
@@ -3012,20 +2993,20 @@
     </row>
     <row r="101" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A101">
-        <v>20</v>
+        <v>250</v>
       </c>
       <c r="B101" t="s">
-        <v>30</v>
+        <v>143</v>
       </c>
       <c r="C101" t="str">
         <f t="shared" si="1"/>
-        <v>SM-L310NZGAEUE</v>
+        <v>SM-R390NZDAEUE</v>
       </c>
       <c r="D101" s="3">
-        <v>8806095660981</v>
+        <v>8806095380353</v>
       </c>
       <c r="E101">
-        <v>126</v>
+        <v>29</v>
       </c>
       <c r="F101" t="s">
         <v>6</v>
@@ -3033,20 +3014,20 @@
     </row>
     <row r="102" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A102">
-        <v>20</v>
+        <v>80</v>
       </c>
       <c r="B102" t="s">
-        <v>31</v>
+        <v>144</v>
       </c>
       <c r="C102" t="str">
         <f t="shared" si="1"/>
-        <v>SM-L320NZSAEUE</v>
+        <v>SM-R390NZSAEUE</v>
       </c>
       <c r="D102" s="3">
-        <v>8806097415756</v>
+        <v>8806095380346</v>
       </c>
       <c r="E102">
-        <v>165</v>
+        <v>29</v>
       </c>
       <c r="F102" t="s">
         <v>6</v>
@@ -3054,233 +3035,233 @@
     </row>
     <row r="103" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A103">
-        <v>5</v>
+        <v>50</v>
       </c>
       <c r="B103" t="s">
-        <v>68</v>
+        <v>11</v>
       </c>
       <c r="C103" t="str">
         <f t="shared" si="1"/>
-        <v>S6003EU</v>
+        <v>EB-P3400XUEGEU</v>
       </c>
       <c r="D103" s="3">
-        <v>622356220743</v>
+        <v>8806094682748</v>
       </c>
       <c r="E103">
-        <v>69</v>
+        <v>16</v>
       </c>
       <c r="F103" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="104" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A104">
-        <v>280</v>
+        <v>5</v>
       </c>
       <c r="B104" t="s">
-        <v>100</v>
+        <v>24</v>
       </c>
       <c r="C104" t="str">
         <f t="shared" si="1"/>
-        <v>DT8270E1</v>
+        <v>SM-L310NZGAEUE</v>
       </c>
       <c r="D104" s="3">
-        <v>3121040084175</v>
+        <v>8806095660981</v>
       </c>
       <c r="E104">
-        <v>34</v>
+        <v>126</v>
       </c>
       <c r="F104" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="105" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A105">
-        <v>180</v>
+        <v>15</v>
       </c>
       <c r="B105" t="s">
-        <v>71</v>
+        <v>25</v>
       </c>
       <c r="C105" t="str">
         <f t="shared" si="1"/>
-        <v>FV2835E0</v>
+        <v>SM-L320NZSAEUE</v>
       </c>
       <c r="D105" s="3">
-        <v>3121040082201</v>
+        <v>8806097415756</v>
       </c>
       <c r="E105">
-        <v>20</v>
+        <v>165</v>
       </c>
       <c r="F105" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="106" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A106">
-        <v>80</v>
+        <v>5</v>
       </c>
       <c r="B106" t="s">
-        <v>109</v>
+        <v>58</v>
       </c>
       <c r="C106" t="str">
         <f t="shared" si="1"/>
-        <v>SV8130E0</v>
+        <v>S6003EU</v>
       </c>
       <c r="D106" s="3">
-        <v>3121040086193</v>
+        <v>622356220743</v>
       </c>
       <c r="E106">
-        <v>99</v>
+        <v>69</v>
       </c>
       <c r="F106" t="s">
-        <v>7</v>
+        <v>145</v>
       </c>
     </row>
     <row r="107" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A107">
-        <v>60</v>
+        <v>230</v>
       </c>
       <c r="B107" t="s">
-        <v>69</v>
+        <v>84</v>
       </c>
       <c r="C107" t="str">
         <f t="shared" si="1"/>
-        <v>FV6812E0</v>
+        <v>DT8270E1</v>
       </c>
       <c r="D107" s="3">
-        <v>3121040077184</v>
+        <v>3121040084175</v>
       </c>
       <c r="E107">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F107" t="s">
-        <v>7</v>
+        <v>145</v>
       </c>
     </row>
     <row r="108" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A108">
-        <v>25</v>
+        <v>160</v>
       </c>
       <c r="B108" t="s">
-        <v>101</v>
+        <v>60</v>
       </c>
       <c r="C108" t="str">
         <f t="shared" si="1"/>
-        <v>FV8066E0</v>
+        <v>FV2835E0</v>
       </c>
       <c r="D108" s="3">
-        <v>3121040086490</v>
+        <v>3121040082201</v>
       </c>
       <c r="E108">
-        <v>48</v>
+        <v>20</v>
       </c>
       <c r="F108" t="s">
-        <v>7</v>
+        <v>145</v>
       </c>
     </row>
     <row r="109" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A109">
-        <v>5</v>
+        <v>80</v>
       </c>
       <c r="B109" t="s">
-        <v>70</v>
+        <v>92</v>
       </c>
       <c r="C109" t="str">
         <f t="shared" si="1"/>
-        <v>KI831E10</v>
+        <v>SV8130E0</v>
       </c>
       <c r="D109" s="3">
-        <v>3045387245955</v>
+        <v>3121040086193</v>
       </c>
       <c r="E109">
-        <v>30</v>
+        <v>99</v>
       </c>
       <c r="F109" t="s">
-        <v>7</v>
+        <v>145</v>
       </c>
     </row>
     <row r="110" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A110">
-        <v>10</v>
+        <v>45</v>
       </c>
       <c r="B110" t="s">
-        <v>102</v>
+        <v>59</v>
       </c>
       <c r="C110" t="str">
         <f t="shared" si="1"/>
-        <v>FV8042E0</v>
+        <v>FV6812E0</v>
       </c>
       <c r="D110" s="3">
-        <v>3121040086469</v>
+        <v>3121040077184</v>
       </c>
       <c r="E110">
-        <v>48</v>
+        <v>35</v>
       </c>
       <c r="F110" t="s">
-        <v>7</v>
+        <v>145</v>
       </c>
     </row>
     <row r="111" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A111">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="B111" t="s">
-        <v>103</v>
+        <v>85</v>
       </c>
       <c r="C111" t="str">
         <f t="shared" si="1"/>
-        <v>FV9E50E0</v>
+        <v>FV8066E0</v>
       </c>
       <c r="D111" s="3">
-        <v>3121040089040</v>
+        <v>3121040086490</v>
       </c>
       <c r="E111">
-        <v>93</v>
+        <v>48</v>
       </c>
       <c r="F111" t="s">
-        <v>7</v>
+        <v>145</v>
       </c>
     </row>
     <row r="112" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A112">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="B112" t="s">
-        <v>110</v>
+        <v>86</v>
       </c>
       <c r="C112" t="str">
         <f t="shared" si="1"/>
-        <v>FV9845E0</v>
+        <v>FV8042E0</v>
       </c>
       <c r="D112" s="3">
-        <v>3121040069271</v>
+        <v>3121040086469</v>
       </c>
       <c r="E112">
-        <v>59</v>
+        <v>48</v>
       </c>
       <c r="F112" t="s">
-        <v>7</v>
+        <v>145</v>
       </c>
     </row>
     <row r="113" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A113">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="B113" t="s">
-        <v>111</v>
+        <v>87</v>
       </c>
       <c r="C113" t="str">
         <f t="shared" si="1"/>
-        <v>FV5718E0</v>
+        <v>FV9E50E0</v>
       </c>
       <c r="D113" s="3">
-        <v>3121040075692</v>
+        <v>3121040089040</v>
       </c>
       <c r="E113">
-        <v>30</v>
+        <v>93</v>
       </c>
       <c r="F113" t="s">
-        <v>7</v>
+        <v>145</v>
       </c>
     </row>
     <row r="114" spans="1:6" x14ac:dyDescent="0.25">
@@ -3288,20 +3269,20 @@
         <v>5</v>
       </c>
       <c r="B114" t="s">
-        <v>112</v>
+        <v>93</v>
       </c>
       <c r="C114" t="str">
         <f t="shared" si="1"/>
-        <v>FV9848E0</v>
+        <v>FV5718E0</v>
       </c>
       <c r="D114" s="3">
-        <v>3121040071526</v>
+        <v>3121040075692</v>
       </c>
       <c r="E114">
-        <v>59</v>
+        <v>30</v>
       </c>
       <c r="F114" t="s">
-        <v>7</v>
+        <v>145</v>
       </c>
     </row>
     <row r="115" spans="1:6" x14ac:dyDescent="0.25">
@@ -3309,49 +3290,49 @@
         <v>5</v>
       </c>
       <c r="B115" t="s">
-        <v>104</v>
+        <v>88</v>
       </c>
       <c r="C115" t="str">
         <f t="shared" si="1"/>
-        <v>FV9852E0</v>
+        <v>FV6872E0</v>
       </c>
       <c r="D115" s="3">
-        <v>3121040095737</v>
+        <v>3121040080184</v>
       </c>
       <c r="E115">
-        <v>65</v>
+        <v>40</v>
       </c>
       <c r="F115" t="s">
-        <v>7</v>
+        <v>145</v>
       </c>
     </row>
     <row r="116" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A116">
-        <v>10</v>
+        <v>45</v>
       </c>
       <c r="B116" t="s">
-        <v>105</v>
+        <v>122</v>
       </c>
       <c r="C116" t="str">
         <f t="shared" si="1"/>
-        <v>FV6872E0</v>
+        <v>FV1713</v>
       </c>
       <c r="D116" s="3">
-        <v>3121040080184</v>
+        <v>3121040067741</v>
       </c>
       <c r="E116">
-        <v>40</v>
+        <v>12.430000000000001</v>
       </c>
       <c r="F116" t="s">
-        <v>7</v>
+        <v>145</v>
       </c>
     </row>
     <row r="117" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A117">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="B117" t="s">
-        <v>106</v>
+        <v>89</v>
       </c>
       <c r="C117" t="str">
         <f t="shared" si="1"/>
@@ -3369,10 +3350,10 @@
     </row>
     <row r="118" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A118">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="B118" t="s">
-        <v>107</v>
+        <v>90</v>
       </c>
       <c r="C118" t="str">
         <f t="shared" si="1"/>
@@ -3390,10 +3371,10 @@
     </row>
     <row r="119" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A119">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="B119" t="s">
-        <v>108</v>
+        <v>91</v>
       </c>
       <c r="C119" t="str">
         <f t="shared" si="1"/>
@@ -3411,23 +3392,23 @@
     </row>
     <row r="120" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A120">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="B120" t="s">
-        <v>153</v>
+        <v>32</v>
       </c>
       <c r="C120" t="str">
         <f t="shared" si="1"/>
-        <v>FV1713</v>
+        <v>178236</v>
       </c>
       <c r="D120" s="3">
-        <v>3121040067741</v>
+        <v>4023103254145</v>
       </c>
       <c r="E120">
-        <v>12.430000000000001</v>
+        <v>155</v>
       </c>
       <c r="F120" t="s">
-        <v>161</v>
+        <v>6</v>
       </c>
     </row>
     <row r="121" spans="1:6" x14ac:dyDescent="0.25">
@@ -3435,17 +3416,16 @@
         <v>80</v>
       </c>
       <c r="B121" t="s">
-        <v>38</v>
-      </c>
-      <c r="C121" t="str">
-        <f t="shared" si="1"/>
-        <v>178236</v>
+        <v>33</v>
+      </c>
+      <c r="C121" s="5" t="s">
+        <v>18</v>
       </c>
       <c r="D121" s="3">
-        <v>4023103254145</v>
+        <v>4023103246584</v>
       </c>
       <c r="E121">
-        <v>155</v>
+        <v>17</v>
       </c>
       <c r="F121" t="s">
         <v>6</v>
@@ -3453,84 +3433,86 @@
     </row>
     <row r="122" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A122">
-        <v>80</v>
+        <v>120</v>
       </c>
       <c r="B122" t="s">
-        <v>39</v>
-      </c>
-      <c r="C122" s="5" t="s">
-        <v>22</v>
+        <v>54</v>
+      </c>
+      <c r="C122" t="str">
+        <f t="shared" si="1"/>
+        <v>BHR6151DE</v>
       </c>
       <c r="D122" s="3">
-        <v>4023103246584</v>
+        <v>6934177787782</v>
       </c>
       <c r="E122">
-        <v>17</v>
+        <v>349</v>
       </c>
       <c r="F122" t="s">
-        <v>6</v>
+        <v>145</v>
       </c>
     </row>
     <row r="123" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A123">
-        <v>600</v>
+        <v>300</v>
       </c>
       <c r="B123" t="s">
-        <v>154</v>
-      </c>
-      <c r="C123" s="5" t="s">
-        <v>22</v>
+        <v>12</v>
+      </c>
+      <c r="C123" t="str">
+        <f t="shared" si="1"/>
+        <v>BHR6942EU</v>
       </c>
       <c r="D123" s="3">
-        <v>4023103233935</v>
+        <v>6941812708347</v>
       </c>
       <c r="E123">
-        <v>75</v>
+        <v>49</v>
       </c>
       <c r="F123" t="s">
-        <v>132</v>
+        <v>145</v>
       </c>
     </row>
     <row r="124" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A124">
-        <v>150</v>
+        <v>15</v>
       </c>
       <c r="B124" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="C124" t="str">
         <f t="shared" si="1"/>
-        <v>BHR6151DE</v>
+        <v>BHR5274GL</v>
       </c>
       <c r="D124" s="3">
-        <v>6934177787782</v>
+        <v>6934177751158</v>
       </c>
       <c r="E124">
-        <v>349</v>
+        <v>95</v>
       </c>
       <c r="F124" t="s">
-        <v>7</v>
+        <v>145</v>
       </c>
     </row>
     <row r="125" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A125">
-        <v>300</v>
+        <v>15</v>
       </c>
       <c r="B125" t="s">
-        <v>15</v>
+        <v>69</v>
       </c>
       <c r="C125" t="str">
         <f t="shared" si="1"/>
-        <v>BHR6942EU</v>
+        <v>BHR08MZEU</v>
       </c>
       <c r="D125" s="3">
-        <v>6941812708347</v>
+        <v>6932554469139</v>
       </c>
       <c r="E125">
-        <v>51</v>
+        <v>123</v>
       </c>
       <c r="F125" t="s">
-        <v>7</v>
+        <v>145</v>
       </c>
     </row>
     <row r="126" spans="1:6" x14ac:dyDescent="0.25">
@@ -3538,143 +3520,143 @@
         <v>50</v>
       </c>
       <c r="B126" t="s">
-        <v>76</v>
+        <v>146</v>
       </c>
       <c r="C126" t="str">
-        <f t="shared" si="1"/>
-        <v>BHR5860EU</v>
+        <f t="shared" ref="C126:C146" si="2">MID(B126,FIND("@",SUBSTITUTE(B126," ","@",LEN(B126)-LEN(SUBSTITUTE(B126," ",""))))+1,LEN(B126))</f>
+        <v>BHR084AEU</v>
       </c>
       <c r="D126" s="3">
-        <v>6934177775345</v>
+        <v>6932554440893</v>
       </c>
       <c r="E126">
-        <v>55</v>
+        <v>102</v>
       </c>
       <c r="F126" t="s">
-        <v>7</v>
+        <v>145</v>
       </c>
     </row>
     <row r="127" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A127">
-        <v>40</v>
+        <v>15</v>
       </c>
       <c r="B127" t="s">
-        <v>81</v>
+        <v>26</v>
       </c>
       <c r="C127" t="str">
-        <f t="shared" ref="C127:C151" si="2">MID(B127,FIND("@",SUBSTITUTE(B127," ","@",LEN(B127)-LEN(SUBSTITUTE(B127," ",""))))+1,LEN(B127))</f>
-        <v>BHR5274GL</v>
+        <f t="shared" si="2"/>
+        <v>BHR9798EU</v>
       </c>
       <c r="D127" s="3">
-        <v>6934177751158</v>
+        <v>6932554403850</v>
       </c>
       <c r="E127">
-        <v>95</v>
+        <v>59</v>
       </c>
       <c r="F127" t="s">
-        <v>7</v>
+        <v>145</v>
       </c>
     </row>
     <row r="128" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A128">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="B128" t="s">
-        <v>82</v>
+        <v>70</v>
       </c>
       <c r="C128" t="str">
         <f t="shared" si="2"/>
-        <v>BHR08MZEU</v>
+        <v>ELA5956EU</v>
       </c>
       <c r="D128" s="3">
-        <v>6932554469139</v>
+        <v>6941948705630</v>
       </c>
       <c r="E128">
-        <v>123</v>
+        <v>210</v>
       </c>
       <c r="F128" t="s">
-        <v>7</v>
+        <v>145</v>
       </c>
     </row>
     <row r="129" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A129">
-        <v>110</v>
+        <v>4000</v>
       </c>
       <c r="B129" t="s">
-        <v>12</v>
+        <v>76</v>
       </c>
       <c r="C129" t="str">
         <f t="shared" si="2"/>
-        <v>BHR8629EU</v>
+        <v>PFJ4191EU</v>
       </c>
       <c r="D129" s="3">
-        <v>6941812786604</v>
+        <v>6941948704916</v>
       </c>
       <c r="E129">
-        <v>90</v>
+        <v>41</v>
       </c>
       <c r="F129" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="130" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A130">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="B130" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="C130" t="str">
         <f t="shared" si="2"/>
-        <v>BHR9798EU</v>
+        <v>BHR08OLGL</v>
       </c>
       <c r="D130" s="3">
-        <v>6932554403850</v>
+        <v>6932554471880</v>
       </c>
       <c r="E130">
-        <v>59</v>
+        <v>16</v>
       </c>
       <c r="F130" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="131" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A131">
-        <v>40</v>
+        <v>30</v>
       </c>
       <c r="B131" t="s">
-        <v>83</v>
+        <v>29</v>
       </c>
       <c r="C131" t="str">
         <f t="shared" si="2"/>
-        <v>ELA5956EU</v>
+        <v>BHR07PSGL</v>
       </c>
       <c r="D131" s="3">
-        <v>6941948705630</v>
+        <v>6932554419813</v>
       </c>
       <c r="E131">
-        <v>210</v>
+        <v>30</v>
       </c>
       <c r="F131" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="132" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A132">
-        <v>300</v>
+        <v>60</v>
       </c>
       <c r="B132" t="s">
-        <v>89</v>
+        <v>77</v>
       </c>
       <c r="C132" t="str">
         <f t="shared" si="2"/>
-        <v>PFJ4191EU</v>
+        <v>BHR9341GL</v>
       </c>
       <c r="D132" s="3">
-        <v>6941948704916</v>
+        <v>6941812774717</v>
       </c>
       <c r="E132">
-        <v>42</v>
+        <v>17</v>
       </c>
       <c r="F132" t="s">
         <v>6</v>
@@ -3682,20 +3664,20 @@
     </row>
     <row r="133" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A133">
-        <v>15</v>
+        <v>60</v>
       </c>
       <c r="B133" t="s">
-        <v>34</v>
+        <v>78</v>
       </c>
       <c r="C133" t="str">
         <f t="shared" si="2"/>
-        <v>BHR08OLGL</v>
+        <v>BHR9333GL</v>
       </c>
       <c r="D133" s="3">
-        <v>6932554471880</v>
+        <v>6941812743669</v>
       </c>
       <c r="E133">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F133" t="s">
         <v>6</v>
@@ -3703,20 +3685,20 @@
     </row>
     <row r="134" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A134">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="B134" t="s">
-        <v>35</v>
+        <v>79</v>
       </c>
       <c r="C134" t="str">
         <f t="shared" si="2"/>
-        <v>BHR07PSGL</v>
+        <v>BHR08O7GL</v>
       </c>
       <c r="D134" s="3">
-        <v>6932554419813</v>
+        <v>6932554471200</v>
       </c>
       <c r="E134">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="F134" t="s">
         <v>6</v>
@@ -3724,20 +3706,20 @@
     </row>
     <row r="135" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A135">
-        <v>65</v>
+        <v>5</v>
       </c>
       <c r="B135" t="s">
-        <v>90</v>
+        <v>30</v>
       </c>
       <c r="C135" t="str">
         <f t="shared" si="2"/>
-        <v>BHR9341GL</v>
+        <v>BHR08PLGL</v>
       </c>
       <c r="D135" s="3">
-        <v>6941812774717</v>
+        <v>6932554473877</v>
       </c>
       <c r="E135">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="F135" t="s">
         <v>6</v>
@@ -3745,20 +3727,20 @@
     </row>
     <row r="136" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A136">
-        <v>65</v>
+        <v>80</v>
       </c>
       <c r="B136" t="s">
-        <v>91</v>
+        <v>7</v>
       </c>
       <c r="C136" t="str">
         <f t="shared" si="2"/>
-        <v>BHR9333GL</v>
+        <v>QBH4380GL</v>
       </c>
       <c r="D136" s="3">
-        <v>6941812743669</v>
+        <v>6941948709218</v>
       </c>
       <c r="E136">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="F136" t="s">
         <v>6</v>
@@ -3766,20 +3748,20 @@
     </row>
     <row r="137" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A137">
-        <v>10</v>
+        <v>100</v>
       </c>
       <c r="B137" t="s">
-        <v>92</v>
+        <v>8</v>
       </c>
       <c r="C137" t="str">
         <f t="shared" si="2"/>
-        <v>BHR8851GL</v>
+        <v>QBH4378GL</v>
       </c>
       <c r="D137" s="3">
-        <v>6941812792155</v>
+        <v>6941948709201</v>
       </c>
       <c r="E137">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c r="F137" t="s">
         <v>6</v>
@@ -3790,17 +3772,17 @@
         <v>40</v>
       </c>
       <c r="B138" t="s">
-        <v>93</v>
+        <v>38</v>
       </c>
       <c r="C138" t="str">
         <f t="shared" si="2"/>
-        <v>BHR08O7GL</v>
+        <v>QBH4265GL</v>
       </c>
       <c r="D138" s="3">
-        <v>6932554471200</v>
+        <v>6941948702042</v>
       </c>
       <c r="E138">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="F138" t="s">
         <v>6</v>
@@ -3811,17 +3793,17 @@
         <v>5</v>
       </c>
       <c r="B139" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C139" t="str">
         <f t="shared" si="2"/>
-        <v>BHR08PLGL</v>
+        <v>QBH4370GL</v>
       </c>
       <c r="D139" s="3">
-        <v>6932554473877</v>
+        <v>6941948709164</v>
       </c>
       <c r="E139">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="F139" t="s">
         <v>6</v>
@@ -3829,20 +3811,20 @@
     </row>
     <row r="140" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A140">
-        <v>80</v>
+        <v>5</v>
       </c>
       <c r="B140" t="s">
-        <v>8</v>
+        <v>40</v>
       </c>
       <c r="C140" t="str">
         <f t="shared" si="2"/>
-        <v>QBH4380GL</v>
+        <v>QBH4372GL</v>
       </c>
       <c r="D140" s="3">
-        <v>6941948709218</v>
+        <v>6941948709171</v>
       </c>
       <c r="E140">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="F140" t="s">
         <v>6</v>
@@ -3850,20 +3832,20 @@
     </row>
     <row r="141" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A141">
-        <v>100</v>
+        <v>70</v>
       </c>
       <c r="B141" t="s">
-        <v>9</v>
+        <v>41</v>
       </c>
       <c r="C141" t="str">
         <f t="shared" si="2"/>
-        <v>QBH4378GL</v>
+        <v>QBH4263GL</v>
       </c>
       <c r="D141" s="3">
-        <v>6941948709201</v>
+        <v>6941948702035</v>
       </c>
       <c r="E141">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="F141" t="s">
         <v>6</v>
@@ -3871,20 +3853,20 @@
     </row>
     <row r="142" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A142">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="B142" t="s">
-        <v>44</v>
+        <v>9</v>
       </c>
       <c r="C142" t="str">
         <f t="shared" si="2"/>
-        <v>QBH4265GL</v>
+        <v>QBH2475GL</v>
       </c>
       <c r="D142" s="3">
-        <v>6941948702042</v>
+        <v>6941948703391</v>
       </c>
       <c r="E142">
-        <v>27</v>
+        <v>38</v>
       </c>
       <c r="F142" t="s">
         <v>6</v>
@@ -3892,20 +3874,20 @@
     </row>
     <row r="143" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A143">
-        <v>10</v>
+        <v>40</v>
       </c>
       <c r="B143" t="s">
-        <v>45</v>
+        <v>71</v>
       </c>
       <c r="C143" t="str">
         <f t="shared" si="2"/>
-        <v>QBH4370GL</v>
+        <v>BHR9036EU</v>
       </c>
       <c r="D143" s="3">
-        <v>6941948709164</v>
+        <v>6941812797013</v>
       </c>
       <c r="E143">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="F143" t="s">
         <v>6</v>
@@ -3913,20 +3895,20 @@
     </row>
     <row r="144" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A144">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="B144" t="s">
-        <v>46</v>
+        <v>13</v>
       </c>
       <c r="C144" t="str">
         <f t="shared" si="2"/>
-        <v>QBH4372GL</v>
+        <v>BHR8811EU</v>
       </c>
       <c r="D144" s="3">
-        <v>6941948709171</v>
+        <v>6941812791868</v>
       </c>
       <c r="E144">
-        <v>27</v>
+        <v>18</v>
       </c>
       <c r="F144" t="s">
         <v>6</v>
@@ -3934,20 +3916,20 @@
     </row>
     <row r="145" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A145">
-        <v>70</v>
+        <v>10</v>
       </c>
       <c r="B145" t="s">
-        <v>47</v>
+        <v>27</v>
       </c>
       <c r="C145" t="str">
         <f t="shared" si="2"/>
-        <v>QBH4263GL</v>
+        <v>BHR5967EU</v>
       </c>
       <c r="D145" s="3">
-        <v>6941948702035</v>
+        <v>6934177763113</v>
       </c>
       <c r="E145">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="F145" t="s">
         <v>6</v>
@@ -3955,132 +3937,24 @@
     </row>
     <row r="146" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A146">
-        <v>50</v>
+        <v>40</v>
       </c>
       <c r="B146" t="s">
-        <v>10</v>
+        <v>72</v>
       </c>
       <c r="C146" t="str">
         <f t="shared" si="2"/>
-        <v>QBH2475GL</v>
+        <v>BHR9099GL</v>
       </c>
       <c r="D146" s="3">
-        <v>6941948703391</v>
+        <v>6941812797853</v>
       </c>
       <c r="E146">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="F146" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="147" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A147">
-        <v>50</v>
-      </c>
-      <c r="B147" t="s">
-        <v>84</v>
-      </c>
-      <c r="C147" t="str">
-        <f t="shared" si="2"/>
-        <v>BHR9036EU</v>
-      </c>
-      <c r="D147" s="3">
-        <v>6941812797013</v>
-      </c>
-      <c r="E147">
-        <v>17</v>
-      </c>
-      <c r="F147" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="148" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A148">
-        <v>50</v>
-      </c>
-      <c r="B148" t="s">
-        <v>16</v>
-      </c>
-      <c r="C148" t="str">
-        <f t="shared" si="2"/>
-        <v>BHR8811EU</v>
-      </c>
-      <c r="D148" s="3">
-        <v>6941812791868</v>
-      </c>
-      <c r="E148">
-        <v>18</v>
-      </c>
-      <c r="F148" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="149" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A149">
-        <v>30</v>
-      </c>
-      <c r="B149" t="s">
-        <v>17</v>
-      </c>
-      <c r="C149" t="str">
-        <f t="shared" si="2"/>
-        <v>BHR9034EU</v>
-      </c>
-      <c r="D149" s="3">
-        <v>6941812796726</v>
-      </c>
-      <c r="E149">
-        <v>23</v>
-      </c>
-      <c r="F149" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="150" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A150">
-        <v>20</v>
-      </c>
-      <c r="B150" t="s">
-        <v>33</v>
-      </c>
-      <c r="C150" t="str">
-        <f t="shared" si="2"/>
-        <v>BHR5967EU</v>
-      </c>
-      <c r="D150" s="3">
-        <v>6934177763113</v>
-      </c>
-      <c r="E150">
-        <v>28</v>
-      </c>
-      <c r="F150" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="151" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A151">
-        <v>45</v>
-      </c>
-      <c r="B151" t="s">
-        <v>85</v>
-      </c>
-      <c r="C151" t="str">
-        <f t="shared" si="2"/>
-        <v>BHR9099GL</v>
-      </c>
-      <c r="D151" s="3">
-        <v>6941812797853</v>
-      </c>
-      <c r="E151">
-        <v>39</v>
-      </c>
-      <c r="F151" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="152" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="D152" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
chnaged and fixed this
</commit_message>
<xml_diff>
--- a/script2/input/ampq.xlsx
+++ b/script2/input/ampq.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Mój dysk\AMPQ\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3361760-1272-484A-A4B8-28875E0E8B47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68B03C25-8D8A-46C8-819A-DE8FF5C983F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3465E9D8-2616-4A3B-901D-12D504620602}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="306" uniqueCount="155">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="260" uniqueCount="132">
   <si>
     <t>QTY</t>
   </si>
@@ -104,9 +104,6 @@
     <t>Xiaomi Redmi Note 15 4G NFC DS 8/256GB Midnight Black MZB0M8FEU</t>
   </si>
   <si>
-    <t>Xiaomi Redmi Pad 2 Pro WIFI 6/128GB Silver VHU6253EU</t>
-  </si>
-  <si>
     <t>Ninja Foodi Power Nutri CB100EU</t>
   </si>
   <si>
@@ -116,9 +113,6 @@
     <t>Samsung Watch 8 40mm BT Silver SM-L320NZSAEUE</t>
   </si>
   <si>
-    <t>Xiaomi Semi-automatic Espresso Machine EU BHR9798EU</t>
-  </si>
-  <si>
     <t>Xiaomi Mi Smart LED Desk Lamp 1S EU BHR5967EU</t>
   </si>
   <si>
@@ -143,9 +137,6 @@
     <t>Apple iPhone 17 256GB Mist Blue MG6L4HX/A</t>
   </si>
   <si>
-    <t>Apple iPhone 17 256GB Lavender MG6M4HX/A</t>
-  </si>
-  <si>
     <t>Midea Microwave Oven 700W MD-MP012MK-WH</t>
   </si>
   <si>
@@ -155,12 +146,6 @@
     <t>Xiaomi Sound Outdoor 30W Blue QBH4265GL</t>
   </si>
   <si>
-    <t>Xiaomi Sound Outdoor 30W Gold GL QBH4370GL</t>
-  </si>
-  <si>
-    <t>Xiaomi Sound Outdoor 30W Green GL QBH4372GL</t>
-  </si>
-  <si>
     <t>Xiaomi Sound Outdoor 30W Red QBH4263GL</t>
   </si>
   <si>
@@ -206,48 +191,24 @@
     <t>Dyson Wash G1 WR01 Cordless Vacuum Blue/Black EU 486236-01</t>
   </si>
   <si>
-    <t>Dyson Vacuum V16 Piston Animal Prussian Blue Copper SV53A 492963-01</t>
-  </si>
-  <si>
     <t>Ninja Air Fryer &amp; Grill 6 in 1 DG551EU</t>
   </si>
   <si>
-    <t>Shark mop parowy Klik'n Flip S6003EU</t>
-  </si>
-  <si>
     <t>Tefal Ultragliss Plus Iron Blue FV6812E0</t>
   </si>
   <si>
     <t>Tefal Express Steam Iron Claret FV2835E0</t>
   </si>
   <si>
-    <t>Xiaomi Redmi 15C 4G 8/256GB Midnight Black MZB0KTPEU</t>
-  </si>
-  <si>
-    <t>Xiaomi Redmi 15C 4G 8/256GB Moonlight Blue MZB0LBMEU</t>
-  </si>
-  <si>
-    <t>Xiaomi Redmi 15C 4G 8/256GB Mint Green MZB0LBVEU</t>
-  </si>
-  <si>
     <t>Logitech Mouse M240 Silent Pink 910-007121</t>
   </si>
   <si>
     <t>Ninja AirFryer 9,5L SL400EU</t>
   </si>
   <si>
-    <t>Ninja AirFryer 9,5l SL400EUWH</t>
-  </si>
-  <si>
     <t>Apple iPhone 17 Pro 256gb Orange MG8H4HX/A</t>
   </si>
   <si>
-    <t>Xiaomi Mi Air Purifier 4 Lite BHR5274GL</t>
-  </si>
-  <si>
-    <t>Xiaomi Mijia Smart Air Purifier 6 EU BHR08MZEU</t>
-  </si>
-  <si>
     <t>Xiaomi TV A Pro 43U 2026 ELA5956EU</t>
   </si>
   <si>
@@ -257,12 +218,6 @@
     <t>Xiaomi Portable Electric Air Compressor 2 Pro BHR9099GL</t>
   </si>
   <si>
-    <t>Apple iPhone 16 128GB Black MYE73HN/A</t>
-  </si>
-  <si>
-    <t>Apple iPhone 16 128GB Teal MYED3HN/A</t>
-  </si>
-  <si>
     <t>Samsung S25 12/128GB BlueBlack SM-S931BZKDEUE</t>
   </si>
   <si>
@@ -296,12 +251,6 @@
     <t>Tefal Puregliss Iron Black&amp;Blue FV8066E0</t>
   </si>
   <si>
-    <t>Tefal Puregliss White/Gold FV8042E0</t>
-  </si>
-  <si>
-    <t>Tefal Ultimate Power Pro Black/Copper FV9E50E0</t>
-  </si>
-  <si>
     <t>Tefal SMART PROTECT PLUS Blue/Silver FV6872E0</t>
   </si>
   <si>
@@ -326,9 +275,6 @@
     <t>Karcher SC 4 EasyFix EU 1.512-630.0</t>
   </si>
   <si>
-    <t>Philips Water Osmosis ADD6920BK/10</t>
-  </si>
-  <si>
     <t>Karcher WV 2 Premium 1.633-426.0</t>
   </si>
   <si>
@@ -356,12 +302,6 @@
     <t>Xiaomi Redmi A7 Pro 4G NFC 4/128GB Black MZB0N5QEU</t>
   </si>
   <si>
-    <t>Xiaomi Redmi Note 15 5G 8/256GB Black MZB0LWMEU</t>
-  </si>
-  <si>
-    <t>(incoming 1-2 days)</t>
-  </si>
-  <si>
     <t>Babyliss Curling iron C338E</t>
   </si>
   <si>
@@ -437,18 +377,9 @@
     <t>Huawei Watch GT 5 Vili-B19F Black Fluoroelastomer Strap 55020DKM</t>
   </si>
   <si>
-    <t>Huawei Watch GT 5 Jana-B19L White Composite Leather Strap 55020DJT</t>
-  </si>
-  <si>
-    <t>Huawei Watch GT 5 Vili-B19W Blue Woven Strap 55020DKH</t>
-  </si>
-  <si>
     <t>Huawei Watch GT 5 Jana-B19M Gold Milanese Strap 55020DJQ</t>
   </si>
   <si>
-    <t>Huawei Watch GT 5 Pro Vili-B29F Black Fluoroelastomer Strap 55020DKD</t>
-  </si>
-  <si>
     <t>Huawei Watch 5 LTE 46mm Rates-L19F Black 55020EWB</t>
   </si>
   <si>
@@ -476,31 +407,31 @@
     <t>(in stock EXW)</t>
   </si>
   <si>
-    <t>Xiaomi Robot Vacuum S40 BHR084AEU</t>
-  </si>
-  <si>
-    <t>(incoming 12.05)</t>
-  </si>
-  <si>
     <t>Apple Pencil 2nd Generation White MXN43ZM/A</t>
   </si>
   <si>
-    <t>Samsung A16 DS 4/128GB Black SM-A165FZKBEUE</t>
-  </si>
-  <si>
-    <t>Samsung A57 8/256GB 5G DS Navy SM-A576BDBDEUE</t>
-  </si>
-  <si>
-    <t>Samsung S26 DS 12/256GB Black SM-S942BZKGEUE</t>
-  </si>
-  <si>
-    <t>Samsung Galaxy S26 Ultra 512GB Black SM-S948BZKGEUE</t>
-  </si>
-  <si>
-    <t>Samsung Tab A11+ 5G 6GB/128GB 11" Grey SM-X236BZAREUE</t>
-  </si>
-  <si>
     <t>Oral-B ELEC TB VITALITY PRO LION KING + TRAVEL CASE</t>
+  </si>
+  <si>
+    <t>Ninja Air Fryer 10,4L Black AF500EU</t>
+  </si>
+  <si>
+    <t>Ninja Multicooker  OL750EU</t>
+  </si>
+  <si>
+    <t>Ninja Slushi Slush-Drink-Maker FS301EU</t>
+  </si>
+  <si>
+    <t>Shark Steam Mop Klik'n Flip S6003EU</t>
+  </si>
+  <si>
+    <t>Philipps OneUp 5000 Series Electric Mop XV5113/01</t>
+  </si>
+  <si>
+    <t>Philips 5500 LatteGo Espresso Machine EP5547/90</t>
+  </si>
+  <si>
+    <t>(incoming 14.05 EXW)</t>
   </si>
 </sst>
 </file>
@@ -890,7 +821,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2A360796-7343-4130-90EE-C427191F85B0}">
-  <dimension ref="A1:F146"/>
+  <dimension ref="A1:F123"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" bestFit="1" customWidth="1"/>
@@ -926,17 +857,17 @@
         <v>14</v>
       </c>
       <c r="B2" t="s">
-        <v>67</v>
+        <v>56</v>
       </c>
       <c r="C2" t="str">
-        <f t="shared" ref="C2:C61" si="0">MID(B2,FIND("@",SUBSTITUTE(B2," ","@",LEN(B2)-LEN(SUBSTITUTE(B2," ",""))))+1,LEN(B2))</f>
+        <f t="shared" ref="C2:C64" si="0">MID(B2,FIND("@",SUBSTITUTE(B2," ","@",LEN(B2)-LEN(SUBSTITUTE(B2," ",""))))+1,LEN(B2))</f>
         <v>MG8H4HX/A</v>
       </c>
       <c r="D2" s="3">
         <v>195950627312</v>
       </c>
       <c r="E2">
-        <v>1065</v>
+        <v>1055</v>
       </c>
       <c r="F2" t="s">
         <v>6</v>
@@ -944,20 +875,20 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="B3" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="C3" t="str">
         <f t="shared" si="0"/>
-        <v>MG6M4HX/A</v>
+        <v>MG6L4HX/A</v>
       </c>
       <c r="D3" s="3">
-        <v>195950644050</v>
+        <v>195950643855</v>
       </c>
       <c r="E3">
-        <v>717</v>
+        <v>716</v>
       </c>
       <c r="F3" t="s">
         <v>6</v>
@@ -965,20 +896,20 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="B4" t="s">
-        <v>34</v>
+        <v>41</v>
       </c>
       <c r="C4" t="str">
         <f t="shared" si="0"/>
-        <v>MG6L4HX/A</v>
+        <v>MG6M4HN/A</v>
       </c>
       <c r="D4" s="3">
-        <v>195950643855</v>
+        <v>195950644043</v>
       </c>
       <c r="E4">
-        <v>717</v>
+        <v>689</v>
       </c>
       <c r="F4" t="s">
         <v>6</v>
@@ -986,20 +917,20 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="B5" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="C5" t="str">
         <f t="shared" si="0"/>
-        <v>MG6M4HN/A</v>
+        <v>MG6L4HN/A</v>
       </c>
       <c r="D5" s="3">
-        <v>195950644043</v>
+        <v>195950643848</v>
       </c>
       <c r="E5">
-        <v>695</v>
+        <v>689</v>
       </c>
       <c r="F5" t="s">
         <v>6</v>
@@ -1007,20 +938,20 @@
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="B6" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="C6" t="str">
         <f t="shared" si="0"/>
-        <v>MG6L4HN/A</v>
+        <v>MG6K4HN/A</v>
       </c>
       <c r="D6" s="3">
-        <v>195950643848</v>
+        <v>195950643640</v>
       </c>
       <c r="E6">
-        <v>695</v>
+        <v>689</v>
       </c>
       <c r="F6" t="s">
         <v>6</v>
@@ -1028,20 +959,20 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7">
-        <v>20</v>
+        <v>195</v>
       </c>
       <c r="B7" t="s">
-        <v>48</v>
+        <v>123</v>
       </c>
       <c r="C7" t="str">
         <f t="shared" si="0"/>
-        <v>MG6K4HN/A</v>
+        <v>MXN43ZM/A</v>
       </c>
       <c r="D7" s="3">
-        <v>195950643640</v>
+        <v>195949690457</v>
       </c>
       <c r="E7">
-        <v>695</v>
+        <v>58</v>
       </c>
       <c r="F7" t="s">
         <v>6</v>
@@ -1049,20 +980,20 @@
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="B8" t="s">
-        <v>73</v>
+        <v>106</v>
       </c>
       <c r="C8" t="str">
         <f t="shared" si="0"/>
-        <v>MYE73HN/A</v>
+        <v>GA09561-GB</v>
       </c>
       <c r="D8" s="3">
-        <v>195949821837</v>
+        <v>840353949737</v>
       </c>
       <c r="E8">
-        <v>579</v>
+        <v>349</v>
       </c>
       <c r="F8" t="s">
         <v>6</v>
@@ -1070,20 +1001,19 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9">
-        <v>30</v>
+        <v>200</v>
       </c>
       <c r="B9" t="s">
-        <v>74</v>
-      </c>
-      <c r="C9" t="str">
-        <f t="shared" si="0"/>
-        <v>MYED3HN/A</v>
+        <v>68</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>18</v>
       </c>
       <c r="D9" s="3">
-        <v>195949822551</v>
+        <v>6941764461062</v>
       </c>
       <c r="E9">
-        <v>579</v>
+        <v>292</v>
       </c>
       <c r="F9" t="s">
         <v>6</v>
@@ -1091,20 +1021,19 @@
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10">
-        <v>195</v>
+        <v>30</v>
       </c>
       <c r="B10" t="s">
-        <v>148</v>
-      </c>
-      <c r="C10" t="str">
-        <f t="shared" si="0"/>
-        <v>MXN43ZM/A</v>
+        <v>65</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>18</v>
       </c>
       <c r="D10" s="3">
-        <v>195949690457</v>
+        <v>6941764482890</v>
       </c>
       <c r="E10">
-        <v>58</v>
+        <v>355</v>
       </c>
       <c r="F10" t="s">
         <v>6</v>
@@ -1112,20 +1041,20 @@
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11">
-        <v>35</v>
+        <v>65</v>
       </c>
       <c r="B11" t="s">
-        <v>126</v>
+        <v>60</v>
       </c>
       <c r="C11" t="str">
         <f t="shared" si="0"/>
-        <v>GA09561-GB</v>
+        <v>SM-S931BZKDEUE</v>
       </c>
       <c r="D11" s="3">
-        <v>840353949737</v>
+        <v>8806095815534</v>
       </c>
       <c r="E11">
-        <v>359</v>
+        <v>490</v>
       </c>
       <c r="F11" t="s">
         <v>6</v>
@@ -1133,19 +1062,20 @@
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12">
-        <v>200</v>
+        <v>20</v>
       </c>
       <c r="B12" t="s">
-        <v>83</v>
-      </c>
-      <c r="C12" s="5" t="s">
-        <v>18</v>
+        <v>19</v>
+      </c>
+      <c r="C12" t="str">
+        <f t="shared" si="0"/>
+        <v>SM-S942BZKHEUE</v>
       </c>
       <c r="D12" s="3">
-        <v>6941764461062</v>
+        <v>8806097827405</v>
       </c>
       <c r="E12">
-        <v>292</v>
+        <v>625</v>
       </c>
       <c r="F12" t="s">
         <v>6</v>
@@ -1153,19 +1083,20 @@
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13">
-        <v>35</v>
+        <v>100</v>
       </c>
       <c r="B13" t="s">
         <v>80</v>
       </c>
-      <c r="C13" s="5" t="s">
-        <v>18</v>
+      <c r="C13" t="str">
+        <f t="shared" si="0"/>
+        <v>MZB0JTEEU</v>
       </c>
       <c r="D13" s="3">
-        <v>6941764482890</v>
+        <v>6932554425432</v>
       </c>
       <c r="E13">
-        <v>355</v>
+        <v>67</v>
       </c>
       <c r="F13" t="s">
         <v>6</v>
@@ -1173,62 +1104,62 @@
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14">
-        <v>500</v>
+        <v>100</v>
       </c>
       <c r="B14" t="s">
-        <v>149</v>
+        <v>81</v>
       </c>
       <c r="C14" t="str">
         <f t="shared" si="0"/>
-        <v>SM-A165FZKBEUE</v>
+        <v>MZB0JRIEU</v>
       </c>
       <c r="D14" s="3">
-        <v>8806095822334</v>
+        <v>6932554425814</v>
       </c>
       <c r="E14">
-        <v>92</v>
+        <v>67</v>
       </c>
       <c r="F14" t="s">
-        <v>147</v>
+        <v>6</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15">
-        <v>100</v>
+        <v>40</v>
       </c>
       <c r="B15" t="s">
-        <v>150</v>
+        <v>82</v>
       </c>
       <c r="C15" t="str">
         <f t="shared" si="0"/>
-        <v>SM-A576BDBDEUE</v>
+        <v>MZB0JSAEU</v>
       </c>
       <c r="D15" s="3">
-        <v>8806099028244</v>
+        <v>6932554424978</v>
       </c>
       <c r="E15">
-        <v>295</v>
+        <v>79</v>
       </c>
       <c r="F15" t="s">
-        <v>107</v>
+        <v>6</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16">
-        <v>75</v>
+        <v>50</v>
       </c>
       <c r="B16" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="C16" t="str">
         <f t="shared" si="0"/>
-        <v>SM-S931BZKDEUE</v>
+        <v>MZB0JSTEU</v>
       </c>
       <c r="D16" s="3">
-        <v>8806095815534</v>
+        <v>6932554425241</v>
       </c>
       <c r="E16">
-        <v>490</v>
+        <v>79</v>
       </c>
       <c r="F16" t="s">
         <v>6</v>
@@ -1236,62 +1167,62 @@
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17">
-        <v>100</v>
+        <v>40</v>
       </c>
       <c r="B17" t="s">
-        <v>75</v>
+        <v>84</v>
       </c>
       <c r="C17" t="str">
         <f t="shared" si="0"/>
-        <v>SM-S931BZKDEUE</v>
+        <v>MZB0JTPEU</v>
       </c>
       <c r="D17" s="3">
-        <v>8806095815534</v>
+        <v>6932554425548</v>
       </c>
       <c r="E17">
-        <v>490</v>
+        <v>79</v>
       </c>
       <c r="F17" t="s">
-        <v>107</v>
+        <v>6</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18">
-        <v>100</v>
+        <v>5</v>
       </c>
       <c r="B18" t="s">
-        <v>151</v>
+        <v>85</v>
       </c>
       <c r="C18" t="str">
         <f t="shared" si="0"/>
-        <v>SM-S942BZKGEUE</v>
+        <v>MZB0N5WEU</v>
       </c>
       <c r="D18" s="3">
-        <v>8806097827467</v>
+        <v>6932554493295</v>
       </c>
       <c r="E18">
-        <v>529</v>
+        <v>79</v>
       </c>
       <c r="F18" t="s">
-        <v>107</v>
+        <v>6</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="B19" t="s">
-        <v>19</v>
+        <v>86</v>
       </c>
       <c r="C19" t="str">
         <f t="shared" si="0"/>
-        <v>SM-S942BZKHEUE</v>
+        <v>MZB0N5TEU</v>
       </c>
       <c r="D19" s="3">
-        <v>8806097827405</v>
+        <v>6932554493264</v>
       </c>
       <c r="E19">
-        <v>625</v>
+        <v>79</v>
       </c>
       <c r="F19" t="s">
         <v>6</v>
@@ -1299,62 +1230,62 @@
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20">
-        <v>100</v>
+        <v>5</v>
       </c>
       <c r="B20" t="s">
-        <v>152</v>
+        <v>87</v>
       </c>
       <c r="C20" t="str">
         <f t="shared" si="0"/>
-        <v>SM-S948BZKGEUE</v>
+        <v>MZB0N5QEU</v>
       </c>
       <c r="D20" s="3">
-        <v>8806097827177</v>
+        <v>6932554493257</v>
       </c>
       <c r="E20">
-        <v>879</v>
+        <v>89</v>
       </c>
       <c r="F20" t="s">
-        <v>107</v>
+        <v>6</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21">
-        <v>120</v>
+        <v>20</v>
       </c>
       <c r="B21" t="s">
-        <v>153</v>
+        <v>21</v>
       </c>
       <c r="C21" t="str">
         <f t="shared" si="0"/>
-        <v>SM-X236BZAREUE</v>
+        <v>MZB0M8FEU</v>
       </c>
       <c r="D21" s="3">
-        <v>8806097854821</v>
+        <v>6932554476274</v>
       </c>
       <c r="E21">
-        <v>179</v>
+        <v>135</v>
       </c>
       <c r="F21" t="s">
-        <v>107</v>
+        <v>6</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A22">
-        <v>100</v>
+        <v>4</v>
       </c>
       <c r="B22" t="s">
-        <v>98</v>
+        <v>105</v>
       </c>
       <c r="C22" t="str">
         <f t="shared" si="0"/>
-        <v>MZB0JTEEU</v>
+        <v>VHU6302EU</v>
       </c>
       <c r="D22" s="3">
-        <v>6932554425432</v>
+        <v>6932554467937</v>
       </c>
       <c r="E22">
-        <v>67</v>
+        <v>185</v>
       </c>
       <c r="F22" t="s">
         <v>6</v>
@@ -1365,17 +1296,17 @@
         <v>100</v>
       </c>
       <c r="B23" t="s">
-        <v>99</v>
+        <v>88</v>
       </c>
       <c r="C23" t="str">
         <f t="shared" si="0"/>
-        <v>MZB0JRIEU</v>
+        <v>C338E</v>
       </c>
       <c r="D23" s="3">
-        <v>6932554425814</v>
+        <v>3030050069419</v>
       </c>
       <c r="E23">
-        <v>67</v>
+        <v>19</v>
       </c>
       <c r="F23" t="s">
         <v>6</v>
@@ -1386,17 +1317,17 @@
         <v>40</v>
       </c>
       <c r="B24" t="s">
-        <v>100</v>
+        <v>89</v>
       </c>
       <c r="C24" t="str">
         <f t="shared" si="0"/>
-        <v>MZB0JSAEU</v>
+        <v>AS962E</v>
       </c>
       <c r="D24" s="3">
-        <v>6932554424978</v>
+        <v>3030050182637</v>
       </c>
       <c r="E24">
-        <v>79</v>
+        <v>37</v>
       </c>
       <c r="F24" t="s">
         <v>6</v>
@@ -1404,20 +1335,20 @@
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A25">
-        <v>50</v>
+        <v>35</v>
       </c>
       <c r="B25" t="s">
-        <v>101</v>
+        <v>90</v>
       </c>
       <c r="C25" t="str">
         <f t="shared" si="0"/>
-        <v>MZB0JSTEU</v>
+        <v>AS960E</v>
       </c>
       <c r="D25" s="3">
-        <v>6932554425241</v>
+        <v>3030050165357</v>
       </c>
       <c r="E25">
-        <v>79</v>
+        <v>41</v>
       </c>
       <c r="F25" t="s">
         <v>6</v>
@@ -1425,20 +1356,20 @@
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A26">
-        <v>40</v>
+        <v>130</v>
       </c>
       <c r="B26" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C26" t="str">
         <f t="shared" si="0"/>
-        <v>MZB0JTPEU</v>
+        <v>TAT6A513</v>
       </c>
       <c r="D26" s="3">
-        <v>6932554425548</v>
+        <v>4242005369782</v>
       </c>
       <c r="E26">
-        <v>79</v>
+        <v>20.680000000000003</v>
       </c>
       <c r="F26" t="s">
         <v>6</v>
@@ -1446,104 +1377,104 @@
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="B27" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="C27" t="str">
         <f t="shared" si="0"/>
-        <v>MZB0N5WEU</v>
+        <v>27F650R</v>
       </c>
       <c r="D27" s="3">
-        <v>6932554493295</v>
+        <v>8592344400261</v>
       </c>
       <c r="E27">
-        <v>79</v>
+        <v>95</v>
       </c>
       <c r="F27" t="s">
-        <v>6</v>
+        <v>122</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A28">
-        <v>5</v>
+        <v>100</v>
       </c>
       <c r="B28" t="s">
-        <v>104</v>
+        <v>66</v>
       </c>
       <c r="C28" t="str">
         <f t="shared" si="0"/>
-        <v>MZB0N5TEU</v>
+        <v>CAF-TF101S-AEUR</v>
       </c>
       <c r="D28" s="3">
-        <v>6932554493264</v>
+        <v>810123673285</v>
       </c>
       <c r="E28">
-        <v>79</v>
+        <v>135</v>
       </c>
       <c r="F28" t="s">
-        <v>6</v>
+        <v>122</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A29">
-        <v>5</v>
+        <v>35</v>
       </c>
       <c r="B29" t="s">
-        <v>105</v>
+        <v>67</v>
       </c>
       <c r="C29" t="str">
         <f t="shared" si="0"/>
-        <v>MZB0N5QEU</v>
+        <v>CAF-DC121-ADER</v>
       </c>
       <c r="D29" s="3">
-        <v>6932554493257</v>
+        <v>810123675227</v>
       </c>
       <c r="E29">
-        <v>89</v>
+        <v>123</v>
       </c>
       <c r="F29" t="s">
-        <v>6</v>
+        <v>122</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="B30" t="s">
-        <v>61</v>
+        <v>50</v>
       </c>
       <c r="C30" t="str">
         <f t="shared" si="0"/>
-        <v>MZB0KTPEU</v>
+        <v>486236-01</v>
       </c>
       <c r="D30" s="3">
-        <v>6932554447144</v>
+        <v>5025155096772</v>
       </c>
       <c r="E30">
-        <v>100</v>
+        <v>309</v>
       </c>
       <c r="F30" t="s">
-        <v>6</v>
+        <v>122</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A31">
-        <v>5</v>
+        <v>90</v>
       </c>
       <c r="B31" t="s">
-        <v>62</v>
+        <v>108</v>
       </c>
       <c r="C31" t="str">
         <f t="shared" si="0"/>
-        <v>MZB0LBMEU</v>
+        <v>W-SO01-0004</v>
       </c>
       <c r="D31" s="3">
-        <v>6932554455927</v>
+        <v>6970135030484</v>
       </c>
       <c r="E31">
-        <v>100</v>
+        <v>6</v>
       </c>
       <c r="F31" t="s">
         <v>6</v>
@@ -1551,83 +1482,83 @@
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A32">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="B32" t="s">
-        <v>63</v>
+        <v>109</v>
       </c>
       <c r="C32" t="str">
         <f t="shared" si="0"/>
-        <v>MZB0LBVEU</v>
+        <v>WG851-11EDR</v>
       </c>
       <c r="D32" s="3">
-        <v>6932554455934</v>
+        <v>6970135033836</v>
       </c>
       <c r="E32">
-        <v>100</v>
+        <v>309</v>
       </c>
       <c r="F32" t="s">
-        <v>6</v>
+        <v>122</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A33">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="B33" t="s">
-        <v>21</v>
+        <v>110</v>
       </c>
       <c r="C33" t="str">
         <f t="shared" si="0"/>
-        <v>MZB0M8FEU</v>
+        <v>WG852-11EDR</v>
       </c>
       <c r="D33" s="3">
-        <v>6932554476274</v>
+        <v>6970135035403</v>
       </c>
       <c r="E33">
-        <v>135</v>
+        <v>239</v>
       </c>
       <c r="F33" t="s">
-        <v>6</v>
+        <v>122</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="B34" t="s">
-        <v>106</v>
+        <v>16</v>
       </c>
       <c r="C34" t="str">
         <f t="shared" si="0"/>
-        <v>MZB0LWMEU</v>
+        <v>B11W6AT</v>
       </c>
       <c r="D34" s="3">
-        <v>6932554469252</v>
+        <v>198828212467</v>
       </c>
       <c r="E34">
-        <v>175</v>
+        <v>110</v>
       </c>
       <c r="F34" t="s">
-        <v>6</v>
+        <v>122</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35">
-        <v>5</v>
+        <v>35</v>
       </c>
       <c r="B35" t="s">
-        <v>22</v>
+        <v>111</v>
       </c>
       <c r="C35" t="str">
         <f t="shared" si="0"/>
-        <v>VHU6253EU</v>
+        <v>55020EYL</v>
       </c>
       <c r="D35" s="3">
-        <v>6932554467319</v>
+        <v>6942103155024</v>
       </c>
       <c r="E35">
-        <v>165</v>
+        <v>89</v>
       </c>
       <c r="F35" t="s">
         <v>6</v>
@@ -1635,20 +1566,20 @@
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A36">
-        <v>5</v>
+        <v>25</v>
       </c>
       <c r="B36" t="s">
-        <v>125</v>
+        <v>112</v>
       </c>
       <c r="C36" t="str">
         <f t="shared" si="0"/>
-        <v>VHU6302EU</v>
+        <v>55020DKM</v>
       </c>
       <c r="D36" s="3">
-        <v>6932554467937</v>
+        <v>6942103132001</v>
       </c>
       <c r="E36">
-        <v>185</v>
+        <v>105</v>
       </c>
       <c r="F36" t="s">
         <v>6</v>
@@ -1656,20 +1587,20 @@
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37">
-        <v>100</v>
+        <v>15</v>
       </c>
       <c r="B37" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="C37" t="str">
         <f t="shared" si="0"/>
-        <v>C338E</v>
+        <v>55020DJQ</v>
       </c>
       <c r="D37" s="3">
-        <v>3030050069419</v>
+        <v>6942103131981</v>
       </c>
       <c r="E37">
-        <v>19</v>
+        <v>144</v>
       </c>
       <c r="F37" t="s">
         <v>6</v>
@@ -1677,20 +1608,20 @@
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38">
-        <v>40</v>
+        <v>5</v>
       </c>
       <c r="B38" t="s">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="C38" t="str">
         <f t="shared" si="0"/>
-        <v>AS962E</v>
+        <v>55020EWB</v>
       </c>
       <c r="D38" s="3">
-        <v>3030050182637</v>
+        <v>6942103154300</v>
       </c>
       <c r="E38">
-        <v>37</v>
+        <v>209</v>
       </c>
       <c r="F38" t="s">
         <v>6</v>
@@ -1698,20 +1629,20 @@
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A39">
-        <v>45</v>
+        <v>20</v>
       </c>
       <c r="B39" t="s">
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="C39" t="str">
         <f t="shared" si="0"/>
-        <v>AS960E</v>
+        <v>55020FTP</v>
       </c>
       <c r="D39" s="3">
-        <v>3030050165357</v>
+        <v>6942103168239</v>
       </c>
       <c r="E39">
-        <v>41</v>
+        <v>189</v>
       </c>
       <c r="F39" t="s">
         <v>6</v>
@@ -1719,20 +1650,20 @@
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A40">
-        <v>136</v>
+        <v>5</v>
       </c>
       <c r="B40" t="s">
-        <v>123</v>
+        <v>116</v>
       </c>
       <c r="C40" t="str">
         <f t="shared" si="0"/>
-        <v>TAT6A513</v>
+        <v>55020FTT</v>
       </c>
       <c r="D40" s="3">
-        <v>4242005369782</v>
+        <v>6942103168192</v>
       </c>
       <c r="E40">
-        <v>20.680000000000003</v>
+        <v>311</v>
       </c>
       <c r="F40" t="s">
         <v>6</v>
@@ -1743,41 +1674,41 @@
         <v>15</v>
       </c>
       <c r="B41" t="s">
-        <v>127</v>
+        <v>91</v>
       </c>
       <c r="C41" t="str">
         <f t="shared" si="0"/>
-        <v>27F650R</v>
+        <v>JBLPBENCORE2EP</v>
       </c>
       <c r="D41" s="3">
-        <v>8592344400261</v>
+        <v>1200130020216</v>
       </c>
       <c r="E41">
-        <v>95</v>
+        <v>185</v>
       </c>
       <c r="F41" t="s">
-        <v>145</v>
+        <v>6</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A42">
-        <v>105</v>
+        <v>30</v>
       </c>
       <c r="B42" t="s">
-        <v>81</v>
+        <v>92</v>
       </c>
       <c r="C42" t="str">
         <f t="shared" si="0"/>
-        <v>CAF-TF101S-AEUR</v>
+        <v>JBLPBENCOREESS2EP</v>
       </c>
       <c r="D42" s="3">
-        <v>810123673285</v>
+        <v>1200130022517</v>
       </c>
       <c r="E42">
-        <v>135</v>
+        <v>132</v>
       </c>
       <c r="F42" t="s">
-        <v>145</v>
+        <v>6</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.25">
@@ -1785,125 +1716,125 @@
         <v>35</v>
       </c>
       <c r="B43" t="s">
-        <v>82</v>
+        <v>79</v>
       </c>
       <c r="C43" t="str">
         <f t="shared" si="0"/>
-        <v>CAF-DC121-ADER</v>
+        <v>1.633-426.0</v>
       </c>
       <c r="D43" s="3">
-        <v>810123675227</v>
+        <v>4054278331393</v>
       </c>
       <c r="E43">
-        <v>123</v>
+        <v>40</v>
       </c>
       <c r="F43" t="s">
-        <v>145</v>
+        <v>122</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A44">
-        <v>30</v>
+        <v>90</v>
       </c>
       <c r="B44" t="s">
-        <v>55</v>
+        <v>46</v>
       </c>
       <c r="C44" t="str">
         <f t="shared" si="0"/>
-        <v>486236-01</v>
+        <v>1.633-701.0</v>
       </c>
       <c r="D44" s="3">
-        <v>5025155096772</v>
+        <v>4054278976600</v>
       </c>
       <c r="E44">
-        <v>309</v>
+        <v>49</v>
       </c>
       <c r="F44" t="s">
-        <v>145</v>
+        <v>122</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="B45" t="s">
-        <v>56</v>
+        <v>44</v>
       </c>
       <c r="C45" t="str">
         <f t="shared" si="0"/>
-        <v>492963-01</v>
+        <v>1.633-514.0</v>
       </c>
       <c r="D45" s="3">
-        <v>5025155114834</v>
+        <v>4054278788616</v>
       </c>
       <c r="E45">
-        <v>565</v>
+        <v>61</v>
       </c>
       <c r="F45" t="s">
-        <v>145</v>
+        <v>122</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A46">
-        <v>100</v>
+        <v>5</v>
       </c>
       <c r="B46" t="s">
-        <v>128</v>
+        <v>45</v>
       </c>
       <c r="C46" t="str">
         <f t="shared" si="0"/>
-        <v>W-SO01-0004</v>
+        <v>1.633-550.0</v>
       </c>
       <c r="D46" s="3">
-        <v>6970135030484</v>
+        <v>4054278348599</v>
       </c>
       <c r="E46">
-        <v>6</v>
+        <v>99</v>
       </c>
       <c r="F46" t="s">
-        <v>6</v>
+        <v>122</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A47">
-        <v>20</v>
+        <v>35</v>
       </c>
       <c r="B47" t="s">
-        <v>129</v>
+        <v>77</v>
       </c>
       <c r="C47" t="str">
         <f t="shared" si="0"/>
-        <v>WG851-11EDR</v>
+        <v>1.513-650.0</v>
       </c>
       <c r="D47" s="3">
-        <v>6970135033836</v>
+        <v>4054278975139</v>
       </c>
       <c r="E47">
-        <v>309</v>
+        <v>114</v>
       </c>
       <c r="F47" t="s">
-        <v>145</v>
+        <v>122</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A48">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="B48" t="s">
-        <v>130</v>
+        <v>78</v>
       </c>
       <c r="C48" t="str">
         <f t="shared" si="0"/>
-        <v>WG852-11EDR</v>
+        <v>1.512-630.0</v>
       </c>
       <c r="D48" s="3">
-        <v>6970135035403</v>
+        <v>4054278991818</v>
       </c>
       <c r="E48">
-        <v>239</v>
+        <v>157</v>
       </c>
       <c r="F48" t="s">
-        <v>145</v>
+        <v>122</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.25">
@@ -1911,38 +1842,38 @@
         <v>10</v>
       </c>
       <c r="B49" t="s">
-        <v>16</v>
+        <v>93</v>
       </c>
       <c r="C49" t="str">
         <f t="shared" si="0"/>
-        <v>B11W6AT</v>
+        <v>1.056-310.0</v>
       </c>
       <c r="D49" s="3">
-        <v>198828212467</v>
+        <v>4054278975153</v>
       </c>
       <c r="E49">
-        <v>110</v>
+        <v>72.600000000000009</v>
       </c>
       <c r="F49" t="s">
-        <v>145</v>
+        <v>122</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A50">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="B50" t="s">
-        <v>131</v>
+        <v>54</v>
       </c>
       <c r="C50" t="str">
         <f t="shared" si="0"/>
-        <v>55020EYL</v>
+        <v>910-007121</v>
       </c>
       <c r="D50" s="3">
-        <v>6942103155024</v>
+        <v>5099206112001</v>
       </c>
       <c r="E50">
-        <v>89</v>
+        <v>13</v>
       </c>
       <c r="F50" t="s">
         <v>6</v>
@@ -1950,20 +1881,20 @@
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A51">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="B51" t="s">
-        <v>132</v>
+        <v>17</v>
       </c>
       <c r="C51" t="str">
         <f t="shared" si="0"/>
-        <v>55020DKM</v>
+        <v>960-001746</v>
       </c>
       <c r="D51" s="3">
-        <v>6942103132001</v>
+        <v>5099206129962</v>
       </c>
       <c r="E51">
-        <v>105</v>
+        <v>81</v>
       </c>
       <c r="F51" t="s">
         <v>6</v>
@@ -1971,20 +1902,20 @@
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A52">
-        <v>5</v>
+        <v>30</v>
       </c>
       <c r="B52" t="s">
-        <v>133</v>
+        <v>47</v>
       </c>
       <c r="C52" t="str">
         <f t="shared" si="0"/>
-        <v>55020DJT</v>
+        <v>941-000112</v>
       </c>
       <c r="D52" s="3">
-        <v>6942103131967</v>
+        <v>5099206057302</v>
       </c>
       <c r="E52">
-        <v>119</v>
+        <v>166</v>
       </c>
       <c r="F52" t="s">
         <v>6</v>
@@ -1992,212 +1923,212 @@
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53">
-        <v>5</v>
+        <v>45</v>
       </c>
       <c r="B53" t="s">
-        <v>134</v>
+        <v>33</v>
       </c>
       <c r="C53" t="str">
         <f t="shared" si="0"/>
-        <v>55020DKH</v>
+        <v>MD-MP012MK-WH</v>
       </c>
       <c r="D53" s="3">
-        <v>6942103132025</v>
+        <v>6944271670965</v>
       </c>
       <c r="E53">
-        <v>119</v>
+        <v>29</v>
       </c>
       <c r="F53" t="s">
-        <v>6</v>
+        <v>122</v>
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="B54" t="s">
-        <v>135</v>
+        <v>55</v>
       </c>
       <c r="C54" t="str">
         <f t="shared" si="0"/>
-        <v>55020DJQ</v>
+        <v>SL400EU</v>
       </c>
       <c r="D54" s="3">
-        <v>6942103131981</v>
+        <v>622356280822</v>
       </c>
       <c r="E54">
-        <v>144</v>
+        <v>121</v>
       </c>
       <c r="F54" t="s">
-        <v>6</v>
+        <v>122</v>
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55">
-        <v>5</v>
+        <v>60</v>
       </c>
       <c r="B55" t="s">
-        <v>136</v>
+        <v>14</v>
       </c>
       <c r="C55" t="str">
         <f t="shared" si="0"/>
-        <v>55020DKD</v>
+        <v>SL451EU</v>
       </c>
       <c r="D55" s="3">
-        <v>6942103132032</v>
+        <v>622356294362</v>
       </c>
       <c r="E55">
-        <v>155</v>
+        <v>145</v>
       </c>
       <c r="F55" t="s">
-        <v>6</v>
+        <v>122</v>
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A56">
-        <v>5</v>
+        <v>90</v>
       </c>
       <c r="B56" t="s">
-        <v>137</v>
+        <v>125</v>
       </c>
       <c r="C56" t="str">
         <f t="shared" si="0"/>
-        <v>55020EWB</v>
+        <v>AF500EU</v>
       </c>
       <c r="D56" s="3">
-        <v>6942103154300</v>
+        <v>622356270373</v>
       </c>
       <c r="E56">
-        <v>209</v>
+        <v>129</v>
       </c>
       <c r="F56" t="s">
-        <v>6</v>
+        <v>122</v>
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A57">
-        <v>30</v>
+        <v>5</v>
       </c>
       <c r="B57" t="s">
-        <v>138</v>
+        <v>34</v>
       </c>
       <c r="C57" t="str">
         <f t="shared" si="0"/>
-        <v>55020FTP</v>
+        <v>AG301EU</v>
       </c>
       <c r="D57" s="3">
-        <v>6942103168239</v>
+        <v>622356232692</v>
       </c>
       <c r="E57">
-        <v>189</v>
+        <v>147</v>
       </c>
       <c r="F57" t="s">
-        <v>6</v>
+        <v>122</v>
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A58">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="B58" t="s">
-        <v>139</v>
+        <v>15</v>
       </c>
       <c r="C58" t="str">
         <f t="shared" si="0"/>
-        <v>55020FTT</v>
+        <v>DZ300EU</v>
       </c>
       <c r="D58" s="3">
-        <v>6942103168192</v>
+        <v>622356322690</v>
       </c>
       <c r="E58">
-        <v>311</v>
+        <v>112</v>
       </c>
       <c r="F58" t="s">
-        <v>6</v>
+        <v>122</v>
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A59">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="B59" t="s">
-        <v>111</v>
+        <v>51</v>
       </c>
       <c r="C59" t="str">
         <f t="shared" si="0"/>
-        <v>JBLPBENCORE2EP</v>
+        <v>DG551EU</v>
       </c>
       <c r="D59" s="3">
-        <v>1200130020216</v>
+        <v>622356293457</v>
       </c>
       <c r="E59">
-        <v>185</v>
+        <v>157</v>
       </c>
       <c r="F59" t="s">
-        <v>6</v>
+        <v>122</v>
       </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A60">
-        <v>50</v>
+        <v>10</v>
       </c>
       <c r="B60" t="s">
-        <v>112</v>
+        <v>126</v>
       </c>
       <c r="C60" t="str">
         <f t="shared" si="0"/>
-        <v>JBLPBENCOREESS2EP</v>
+        <v>OL750EU</v>
       </c>
       <c r="D60" s="3">
-        <v>1200130022517</v>
+        <v>622356245050</v>
       </c>
       <c r="E60">
-        <v>132</v>
+        <v>205</v>
       </c>
       <c r="F60" t="s">
-        <v>6</v>
+        <v>122</v>
       </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A61">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="B61" t="s">
-        <v>97</v>
+        <v>127</v>
       </c>
       <c r="C61" t="str">
         <f t="shared" si="0"/>
-        <v>1.633-426.0</v>
+        <v>FS301EU</v>
       </c>
       <c r="D61" s="3">
-        <v>4054278331393</v>
+        <v>622356294072</v>
       </c>
       <c r="E61">
-        <v>40</v>
+        <v>169</v>
       </c>
       <c r="F61" t="s">
-        <v>145</v>
+        <v>122</v>
       </c>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A62">
-        <v>90</v>
+        <v>15</v>
       </c>
       <c r="B62" t="s">
-        <v>51</v>
+        <v>22</v>
       </c>
       <c r="C62" t="str">
-        <f t="shared" ref="C62:C125" si="1">MID(B62,FIND("@",SUBSTITUTE(B62," ","@",LEN(B62)-LEN(SUBSTITUTE(B62," ",""))))+1,LEN(B62))</f>
-        <v>1.633-701.0</v>
+        <f t="shared" si="0"/>
+        <v>CB100EU</v>
       </c>
       <c r="D62" s="3">
-        <v>4054278976600</v>
+        <v>622356236775</v>
       </c>
       <c r="E62">
-        <v>49</v>
+        <v>85</v>
       </c>
       <c r="F62" t="s">
-        <v>145</v>
+        <v>122</v>
       </c>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.25">
@@ -2205,122 +2136,122 @@
         <v>5</v>
       </c>
       <c r="B63" t="s">
-        <v>49</v>
+        <v>20</v>
       </c>
       <c r="C63" t="str">
-        <f t="shared" si="1"/>
-        <v>1.633-514.0</v>
+        <f t="shared" si="0"/>
+        <v>ES701EU</v>
       </c>
       <c r="D63" s="3">
-        <v>4054278788616</v>
+        <v>622356289825</v>
       </c>
       <c r="E63">
-        <v>61</v>
+        <v>410</v>
       </c>
       <c r="F63" t="s">
-        <v>145</v>
+        <v>122</v>
       </c>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A64">
-        <v>10</v>
+        <v>190</v>
       </c>
       <c r="B64" t="s">
-        <v>50</v>
+        <v>94</v>
       </c>
       <c r="C64" t="str">
-        <f t="shared" si="1"/>
-        <v>1.633-550.0</v>
+        <f t="shared" si="0"/>
+        <v>426967</v>
       </c>
       <c r="D64" s="3">
-        <v>4054278348599</v>
+        <v>4210201426967</v>
       </c>
       <c r="E64">
-        <v>99</v>
+        <v>15.400000000000002</v>
       </c>
       <c r="F64" t="s">
-        <v>145</v>
+        <v>6</v>
       </c>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A65">
-        <v>35</v>
+        <v>190</v>
       </c>
       <c r="B65" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C65" t="str">
-        <f t="shared" si="1"/>
-        <v>1.513-650.0</v>
+        <f t="shared" ref="C65:C123" si="1">MID(B65,FIND("@",SUBSTITUTE(B65," ","@",LEN(B65)-LEN(SUBSTITUTE(B65," ",""))))+1,LEN(B65))</f>
+        <v>446392</v>
       </c>
       <c r="D65" s="3">
-        <v>4054278975139</v>
+        <v>4210201446392</v>
       </c>
       <c r="E65">
-        <v>114</v>
+        <v>15.400000000000002</v>
       </c>
       <c r="F65" t="s">
-        <v>145</v>
+        <v>6</v>
       </c>
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A66">
-        <v>20</v>
+        <v>120</v>
       </c>
       <c r="B66" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C66" t="str">
         <f t="shared" si="1"/>
-        <v>1.512-630.0</v>
+        <v>D103</v>
       </c>
       <c r="D66" s="3">
-        <v>4054278991818</v>
+        <v>4210201432227</v>
       </c>
       <c r="E66">
-        <v>157</v>
+        <v>29.150000000000002</v>
       </c>
       <c r="F66" t="s">
-        <v>145</v>
+        <v>6</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A67">
-        <v>10</v>
+        <v>50</v>
       </c>
       <c r="B67" t="s">
-        <v>113</v>
+        <v>97</v>
       </c>
       <c r="C67" t="str">
         <f t="shared" si="1"/>
-        <v>1.056-310.0</v>
+        <v>914170</v>
       </c>
       <c r="D67" s="3">
-        <v>4054278975153</v>
+        <v>8001090914415</v>
       </c>
       <c r="E67">
-        <v>72.600000000000009</v>
+        <v>24.750000000000004</v>
       </c>
       <c r="F67" t="s">
-        <v>145</v>
+        <v>6</v>
       </c>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A68">
-        <v>40</v>
+        <v>80</v>
       </c>
       <c r="B68" t="s">
-        <v>64</v>
+        <v>98</v>
       </c>
       <c r="C68" t="str">
         <f t="shared" si="1"/>
-        <v>910-007121</v>
+        <v>3216721</v>
       </c>
       <c r="D68" s="3">
-        <v>5099206112001</v>
+        <v>8001090914941</v>
       </c>
       <c r="E68">
-        <v>13</v>
+        <v>24.750000000000004</v>
       </c>
       <c r="F68" t="s">
         <v>6</v>
@@ -2328,20 +2259,19 @@
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A69">
-        <v>20</v>
+        <v>100</v>
       </c>
       <c r="B69" t="s">
-        <v>17</v>
-      </c>
-      <c r="C69" t="str">
-        <f t="shared" si="1"/>
-        <v>960-001746</v>
+        <v>99</v>
+      </c>
+      <c r="C69" s="5" t="s">
+        <v>18</v>
       </c>
       <c r="D69" s="3">
-        <v>5099206129962</v>
+        <v>8006530069373</v>
       </c>
       <c r="E69">
-        <v>81</v>
+        <v>58.300000000000004</v>
       </c>
       <c r="F69" t="s">
         <v>6</v>
@@ -2349,20 +2279,19 @@
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A70">
-        <v>30</v>
+        <v>140</v>
       </c>
       <c r="B70" t="s">
-        <v>52</v>
-      </c>
-      <c r="C70" t="str">
-        <f t="shared" si="1"/>
-        <v>941-000112</v>
+        <v>100</v>
+      </c>
+      <c r="C70" s="5" t="s">
+        <v>18</v>
       </c>
       <c r="D70" s="3">
-        <v>5099206057302</v>
+        <v>8006540773307</v>
       </c>
       <c r="E70">
-        <v>166</v>
+        <v>17.380000000000003</v>
       </c>
       <c r="F70" t="s">
         <v>6</v>
@@ -2370,209 +2299,204 @@
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A71">
-        <v>45</v>
+        <v>135</v>
       </c>
       <c r="B71" t="s">
-        <v>36</v>
-      </c>
-      <c r="C71" t="str">
-        <f t="shared" si="1"/>
-        <v>MD-MP012MK-WH</v>
+        <v>124</v>
+      </c>
+      <c r="C71" s="5" t="s">
+        <v>18</v>
       </c>
       <c r="D71" s="3">
-        <v>6944271670965</v>
+        <v>8700216297172</v>
       </c>
       <c r="E71">
-        <v>29</v>
+        <v>17.380000000000003</v>
       </c>
       <c r="F71" t="s">
-        <v>145</v>
+        <v>6</v>
       </c>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A72">
-        <v>20</v>
+        <v>200</v>
       </c>
       <c r="B72" t="s">
-        <v>65</v>
+        <v>48</v>
       </c>
       <c r="C72" t="str">
         <f t="shared" si="1"/>
-        <v>SL400EU</v>
+        <v>NA352/00</v>
       </c>
       <c r="D72" s="3">
-        <v>622356280822</v>
+        <v>8720389032998</v>
       </c>
       <c r="E72">
-        <v>121</v>
+        <v>93</v>
       </c>
       <c r="F72" t="s">
-        <v>145</v>
+        <v>122</v>
       </c>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A73">
+        <v>50</v>
+      </c>
+      <c r="B73" t="s">
         <v>10</v>
       </c>
-      <c r="B73" t="s">
-        <v>66</v>
-      </c>
       <c r="C73" t="str">
         <f t="shared" si="1"/>
-        <v>SL400EUWH</v>
+        <v>BRI940/00</v>
       </c>
       <c r="D73" s="3">
-        <v>622356303866</v>
+        <v>8720689020206</v>
       </c>
       <c r="E73">
-        <v>130</v>
+        <v>199</v>
       </c>
       <c r="F73" t="s">
-        <v>145</v>
+        <v>122</v>
       </c>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A74">
-        <v>60</v>
+        <v>200</v>
       </c>
       <c r="B74" t="s">
-        <v>14</v>
+        <v>129</v>
       </c>
       <c r="C74" t="str">
         <f t="shared" si="1"/>
-        <v>SL451EU</v>
+        <v>XV5113/01</v>
       </c>
       <c r="D74" s="3">
-        <v>622356294362</v>
+        <v>8720389035975</v>
       </c>
       <c r="E74">
-        <v>145</v>
+        <v>118</v>
       </c>
       <c r="F74" t="s">
-        <v>145</v>
+        <v>131</v>
       </c>
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A75">
-        <v>5</v>
+        <v>48</v>
       </c>
       <c r="B75" t="s">
-        <v>37</v>
+        <v>130</v>
       </c>
       <c r="C75" t="str">
         <f t="shared" si="1"/>
-        <v>AG301EU</v>
+        <v>EP5547/90</v>
       </c>
       <c r="D75" s="3">
-        <v>622356232692</v>
+        <v>8720389032370</v>
       </c>
       <c r="E75">
-        <v>147</v>
+        <v>432</v>
       </c>
       <c r="F75" t="s">
-        <v>145</v>
+        <v>131</v>
       </c>
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A76">
+        <v>40</v>
+      </c>
+      <c r="B76" t="s">
+        <v>104</v>
+      </c>
+      <c r="C76" t="str">
+        <f t="shared" si="1"/>
+        <v>BHD302/10</v>
+      </c>
+      <c r="D76" s="3">
+        <v>8710103959533</v>
+      </c>
+      <c r="E76">
         <v>10</v>
       </c>
-      <c r="B76" t="s">
-        <v>15</v>
-      </c>
-      <c r="C76" t="str">
-        <f t="shared" si="1"/>
-        <v>DZ300EU</v>
-      </c>
-      <c r="D76" s="3">
-        <v>622356322690</v>
-      </c>
-      <c r="E76">
-        <v>112</v>
-      </c>
       <c r="F76" t="s">
-        <v>145</v>
+        <v>6</v>
       </c>
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A77">
-        <v>5</v>
+        <v>30</v>
       </c>
       <c r="B77" t="s">
-        <v>57</v>
-      </c>
-      <c r="C77" t="str">
-        <f t="shared" si="1"/>
-        <v>DG551EU</v>
+        <v>37</v>
+      </c>
+      <c r="C77" s="5" t="s">
+        <v>18</v>
       </c>
       <c r="D77" s="3">
-        <v>622356293457</v>
+        <v>6941764428546</v>
       </c>
       <c r="E77">
-        <v>157</v>
+        <v>9</v>
       </c>
       <c r="F77" t="s">
-        <v>145</v>
+        <v>6</v>
       </c>
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A78">
-        <v>5</v>
+        <v>80</v>
       </c>
       <c r="B78" t="s">
-        <v>20</v>
-      </c>
-      <c r="C78" t="str">
-        <f t="shared" si="1"/>
-        <v>ES701EU</v>
+        <v>38</v>
+      </c>
+      <c r="C78" s="5" t="s">
+        <v>18</v>
       </c>
       <c r="D78" s="3">
-        <v>622356289825</v>
+        <v>6941764467194</v>
       </c>
       <c r="E78">
-        <v>410</v>
+        <v>13</v>
       </c>
       <c r="F78" t="s">
-        <v>145</v>
+        <v>6</v>
       </c>
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A79">
-        <v>15</v>
+        <v>100</v>
       </c>
       <c r="B79" t="s">
-        <v>23</v>
-      </c>
-      <c r="C79" t="str">
-        <f t="shared" si="1"/>
-        <v>CB100EU</v>
+        <v>39</v>
+      </c>
+      <c r="C79" s="5" t="s">
+        <v>18</v>
       </c>
       <c r="D79" s="3">
-        <v>622356236775</v>
+        <v>6941764432994</v>
       </c>
       <c r="E79">
-        <v>85</v>
+        <v>19</v>
       </c>
       <c r="F79" t="s">
-        <v>145</v>
+        <v>6</v>
       </c>
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A80">
-        <v>200</v>
+        <v>10</v>
       </c>
       <c r="B80" t="s">
-        <v>114</v>
-      </c>
-      <c r="C80" t="str">
-        <f t="shared" si="1"/>
-        <v>426967</v>
+        <v>40</v>
+      </c>
+      <c r="C80" s="5" t="s">
+        <v>18</v>
       </c>
       <c r="D80" s="3">
-        <v>4210201426967</v>
+        <v>6941764483408</v>
       </c>
       <c r="E80">
-        <v>15.400000000000002</v>
+        <v>39</v>
       </c>
       <c r="F80" t="s">
         <v>6</v>
@@ -2580,20 +2504,20 @@
     </row>
     <row r="81" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A81">
-        <v>200</v>
+        <v>40</v>
       </c>
       <c r="B81" t="s">
-        <v>115</v>
+        <v>29</v>
       </c>
       <c r="C81" t="str">
         <f t="shared" si="1"/>
-        <v>446392</v>
+        <v>MB4700</v>
       </c>
       <c r="D81" s="3">
-        <v>4210201446392</v>
+        <v>4008496942060</v>
       </c>
       <c r="E81">
-        <v>15.400000000000002</v>
+        <v>22</v>
       </c>
       <c r="F81" t="s">
         <v>6</v>
@@ -2601,41 +2525,41 @@
     </row>
     <row r="82" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A82">
-        <v>120</v>
+        <v>30</v>
       </c>
       <c r="B82" t="s">
-        <v>116</v>
+        <v>101</v>
       </c>
       <c r="C82" t="str">
         <f t="shared" si="1"/>
-        <v>D103</v>
+        <v>26510-56</v>
       </c>
       <c r="D82" s="3">
-        <v>4210201432227</v>
+        <v>5038061142860</v>
       </c>
       <c r="E82">
-        <v>29.150000000000002</v>
+        <v>38.5</v>
       </c>
       <c r="F82" t="s">
-        <v>6</v>
+        <v>122</v>
       </c>
     </row>
     <row r="83" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A83">
-        <v>50</v>
+        <v>1200</v>
       </c>
       <c r="B83" t="s">
         <v>117</v>
       </c>
       <c r="C83" t="str">
         <f t="shared" si="1"/>
-        <v>914170</v>
+        <v>EI-T5600BBEGEU</v>
       </c>
       <c r="D83" s="3">
-        <v>8001090914415</v>
+        <v>8806095039893</v>
       </c>
       <c r="E83">
-        <v>24.750000000000004</v>
+        <v>12</v>
       </c>
       <c r="F83" t="s">
         <v>6</v>
@@ -2643,20 +2567,20 @@
     </row>
     <row r="84" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A84">
-        <v>80</v>
+        <v>650</v>
       </c>
       <c r="B84" t="s">
         <v>118</v>
       </c>
       <c r="C84" t="str">
         <f t="shared" si="1"/>
-        <v>3216721</v>
+        <v>EI-T5600BWEGEU</v>
       </c>
       <c r="D84" s="3">
-        <v>8001090914941</v>
+        <v>8806095039824</v>
       </c>
       <c r="E84">
-        <v>24.750000000000004</v>
+        <v>12</v>
       </c>
       <c r="F84" t="s">
         <v>6</v>
@@ -2664,19 +2588,20 @@
     </row>
     <row r="85" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A85">
-        <v>110</v>
+        <v>40</v>
       </c>
       <c r="B85" t="s">
-        <v>119</v>
-      </c>
-      <c r="C85" s="5" t="s">
-        <v>18</v>
+        <v>11</v>
+      </c>
+      <c r="C85" t="str">
+        <f t="shared" si="1"/>
+        <v>EB-P3400XUEGEU</v>
       </c>
       <c r="D85" s="3">
-        <v>8006530069373</v>
+        <v>8806094682748</v>
       </c>
       <c r="E85">
-        <v>58.300000000000004</v>
+        <v>16</v>
       </c>
       <c r="F85" t="s">
         <v>6</v>
@@ -2684,19 +2609,20 @@
     </row>
     <row r="86" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A86">
-        <v>140</v>
+        <v>440</v>
       </c>
       <c r="B86" t="s">
-        <v>120</v>
-      </c>
-      <c r="C86" s="5" t="s">
-        <v>18</v>
+        <v>119</v>
+      </c>
+      <c r="C86" t="str">
+        <f t="shared" si="1"/>
+        <v>SM-R390NZAAMEA</v>
       </c>
       <c r="D86" s="3">
-        <v>8006540773307</v>
+        <v>8806095380384</v>
       </c>
       <c r="E86">
-        <v>17.380000000000003</v>
+        <v>29</v>
       </c>
       <c r="F86" t="s">
         <v>6</v>
@@ -2704,19 +2630,20 @@
     </row>
     <row r="87" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A87">
-        <v>138</v>
+        <v>250</v>
       </c>
       <c r="B87" t="s">
-        <v>154</v>
-      </c>
-      <c r="C87" s="5" t="s">
-        <v>18</v>
+        <v>120</v>
+      </c>
+      <c r="C87" t="str">
+        <f t="shared" si="1"/>
+        <v>SM-R390NZDAEUE</v>
       </c>
       <c r="D87" s="3">
-        <v>8700216297172</v>
+        <v>8806095380353</v>
       </c>
       <c r="E87">
-        <v>17.380000000000003</v>
+        <v>29</v>
       </c>
       <c r="F87" t="s">
         <v>6</v>
@@ -2724,62 +2651,62 @@
     </row>
     <row r="88" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A88">
-        <v>200</v>
+        <v>80</v>
       </c>
       <c r="B88" t="s">
-        <v>53</v>
+        <v>121</v>
       </c>
       <c r="C88" t="str">
         <f t="shared" si="1"/>
-        <v>NA352/00</v>
+        <v>SM-R390NZSAEUE</v>
       </c>
       <c r="D88" s="3">
-        <v>8720389032998</v>
+        <v>8806095380346</v>
       </c>
       <c r="E88">
-        <v>93</v>
+        <v>29</v>
       </c>
       <c r="F88" t="s">
-        <v>145</v>
+        <v>6</v>
       </c>
     </row>
     <row r="89" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A89">
-        <v>50</v>
+        <v>5</v>
       </c>
       <c r="B89" t="s">
-        <v>10</v>
+        <v>23</v>
       </c>
       <c r="C89" t="str">
         <f t="shared" si="1"/>
-        <v>BRI940/00</v>
+        <v>SM-L310NZGAEUE</v>
       </c>
       <c r="D89" s="3">
-        <v>8720689020206</v>
+        <v>8806095660981</v>
       </c>
       <c r="E89">
-        <v>199</v>
+        <v>126</v>
       </c>
       <c r="F89" t="s">
-        <v>145</v>
+        <v>6</v>
       </c>
     </row>
     <row r="90" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A90">
-        <v>40</v>
+        <v>10</v>
       </c>
       <c r="B90" t="s">
-        <v>124</v>
+        <v>24</v>
       </c>
       <c r="C90" t="str">
         <f t="shared" si="1"/>
-        <v>BHD302/10</v>
+        <v>SM-L320NZSAEUE</v>
       </c>
       <c r="D90" s="3">
-        <v>8710103959533</v>
+        <v>8806097415756</v>
       </c>
       <c r="E90">
-        <v>10</v>
+        <v>165</v>
       </c>
       <c r="F90" t="s">
         <v>6</v>
@@ -2790,202 +2717,206 @@
         <v>5</v>
       </c>
       <c r="B91" t="s">
-        <v>96</v>
+        <v>128</v>
       </c>
       <c r="C91" t="str">
         <f t="shared" si="1"/>
-        <v>ADD6920BK/10</v>
+        <v>S6003EU</v>
       </c>
       <c r="D91" s="3">
-        <v>4895244610766</v>
+        <v>622356220743</v>
       </c>
       <c r="E91">
-        <v>280</v>
+        <v>69</v>
       </c>
       <c r="F91" t="s">
-        <v>145</v>
+        <v>122</v>
       </c>
     </row>
     <row r="92" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A92">
-        <v>30</v>
+        <v>180</v>
       </c>
       <c r="B92" t="s">
-        <v>42</v>
-      </c>
-      <c r="C92" s="5" t="s">
-        <v>18</v>
+        <v>69</v>
+      </c>
+      <c r="C92" t="str">
+        <f t="shared" si="1"/>
+        <v>DT8270E1</v>
       </c>
       <c r="D92" s="3">
-        <v>6941764428546</v>
+        <v>3121040084175</v>
       </c>
       <c r="E92">
-        <v>9</v>
+        <v>34</v>
       </c>
       <c r="F92" t="s">
-        <v>6</v>
+        <v>122</v>
       </c>
     </row>
     <row r="93" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A93">
-        <v>80</v>
+        <v>160</v>
       </c>
       <c r="B93" t="s">
-        <v>43</v>
-      </c>
-      <c r="C93" s="5" t="s">
-        <v>18</v>
+        <v>53</v>
+      </c>
+      <c r="C93" t="str">
+        <f t="shared" si="1"/>
+        <v>FV2835E0</v>
       </c>
       <c r="D93" s="3">
-        <v>6941764467194</v>
+        <v>3121040082201</v>
       </c>
       <c r="E93">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="F93" t="s">
-        <v>6</v>
+        <v>122</v>
       </c>
     </row>
     <row r="94" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A94">
-        <v>120</v>
+        <v>80</v>
       </c>
       <c r="B94" t="s">
-        <v>44</v>
-      </c>
-      <c r="C94" s="5" t="s">
-        <v>18</v>
+        <v>75</v>
+      </c>
+      <c r="C94" t="str">
+        <f t="shared" si="1"/>
+        <v>SV8130E0</v>
       </c>
       <c r="D94" s="3">
-        <v>6941764432994</v>
+        <v>3121040086193</v>
       </c>
       <c r="E94">
-        <v>19</v>
+        <v>99</v>
       </c>
       <c r="F94" t="s">
-        <v>6</v>
+        <v>122</v>
       </c>
     </row>
     <row r="95" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A95">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="B95" t="s">
-        <v>45</v>
-      </c>
-      <c r="C95" s="5" t="s">
-        <v>18</v>
+        <v>52</v>
+      </c>
+      <c r="C95" t="str">
+        <f t="shared" si="1"/>
+        <v>FV6812E0</v>
       </c>
       <c r="D95" s="3">
-        <v>6941764483408</v>
+        <v>3121040077184</v>
       </c>
       <c r="E95">
-        <v>39</v>
+        <v>35</v>
       </c>
       <c r="F95" t="s">
-        <v>6</v>
+        <v>122</v>
       </c>
     </row>
     <row r="96" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A96">
-        <v>40</v>
+        <v>20</v>
       </c>
       <c r="B96" t="s">
-        <v>31</v>
+        <v>70</v>
       </c>
       <c r="C96" t="str">
         <f t="shared" si="1"/>
-        <v>MB4700</v>
+        <v>FV8066E0</v>
       </c>
       <c r="D96" s="3">
-        <v>4008496942060</v>
+        <v>3121040086490</v>
       </c>
       <c r="E96">
-        <v>22</v>
+        <v>48</v>
       </c>
       <c r="F96" t="s">
-        <v>6</v>
+        <v>122</v>
       </c>
     </row>
     <row r="97" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A97">
+        <v>5</v>
+      </c>
+      <c r="B97" t="s">
+        <v>76</v>
+      </c>
+      <c r="C97" t="str">
+        <f t="shared" si="1"/>
+        <v>FV5718E0</v>
+      </c>
+      <c r="D97" s="3">
+        <v>3121040075692</v>
+      </c>
+      <c r="E97">
         <v>30</v>
       </c>
-      <c r="B97" t="s">
-        <v>121</v>
-      </c>
-      <c r="C97" t="str">
-        <f t="shared" si="1"/>
-        <v>26510-56</v>
-      </c>
-      <c r="D97" s="3">
-        <v>5038061142860</v>
-      </c>
-      <c r="E97">
-        <v>38.5</v>
-      </c>
       <c r="F97" t="s">
-        <v>145</v>
+        <v>122</v>
       </c>
     </row>
     <row r="98" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A98">
-        <v>1600</v>
+        <v>5</v>
       </c>
       <c r="B98" t="s">
-        <v>140</v>
+        <v>71</v>
       </c>
       <c r="C98" t="str">
         <f t="shared" si="1"/>
-        <v>EI-T5600BBEGEU</v>
+        <v>FV6872E0</v>
       </c>
       <c r="D98" s="3">
-        <v>8806095039893</v>
+        <v>3121040080184</v>
       </c>
       <c r="E98">
-        <v>12</v>
+        <v>40</v>
       </c>
       <c r="F98" t="s">
-        <v>6</v>
+        <v>122</v>
       </c>
     </row>
     <row r="99" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A99">
-        <v>850</v>
+        <v>45</v>
       </c>
       <c r="B99" t="s">
-        <v>141</v>
+        <v>102</v>
       </c>
       <c r="C99" t="str">
         <f t="shared" si="1"/>
-        <v>EI-T5600BWEGEU</v>
+        <v>FV1713</v>
       </c>
       <c r="D99" s="3">
-        <v>8806095039824</v>
+        <v>3121040067741</v>
       </c>
       <c r="E99">
-        <v>12</v>
+        <v>12.430000000000001</v>
       </c>
       <c r="F99" t="s">
-        <v>6</v>
+        <v>122</v>
       </c>
     </row>
     <row r="100" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A100">
-        <v>450</v>
+        <v>20</v>
       </c>
       <c r="B100" t="s">
-        <v>142</v>
+        <v>72</v>
       </c>
       <c r="C100" t="str">
         <f t="shared" si="1"/>
-        <v>SM-R390NZAAMEA</v>
+        <v>BC50D4V0</v>
       </c>
       <c r="D100" s="3">
-        <v>8806095380384</v>
+        <v>3121040092439</v>
       </c>
       <c r="E100">
-        <v>29</v>
+        <v>13</v>
       </c>
       <c r="F100" t="s">
         <v>6</v>
@@ -2993,20 +2924,20 @@
     </row>
     <row r="101" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A101">
-        <v>250</v>
+        <v>20</v>
       </c>
       <c r="B101" t="s">
-        <v>143</v>
+        <v>73</v>
       </c>
       <c r="C101" t="str">
         <f t="shared" si="1"/>
-        <v>SM-R390NZDAEUE</v>
+        <v>PP1803V0</v>
       </c>
       <c r="D101" s="3">
-        <v>8806095380353</v>
+        <v>3121040095317</v>
       </c>
       <c r="E101">
-        <v>29</v>
+        <v>10</v>
       </c>
       <c r="F101" t="s">
         <v>6</v>
@@ -3014,20 +2945,20 @@
     </row>
     <row r="102" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A102">
-        <v>80</v>
+        <v>20</v>
       </c>
       <c r="B102" t="s">
-        <v>144</v>
+        <v>74</v>
       </c>
       <c r="C102" t="str">
         <f t="shared" si="1"/>
-        <v>SM-R390NZSAEUE</v>
+        <v>PP1806</v>
       </c>
       <c r="D102" s="3">
-        <v>8806095380346</v>
+        <v>3121040095355</v>
       </c>
       <c r="E102">
-        <v>29</v>
+        <v>10</v>
       </c>
       <c r="F102" t="s">
         <v>6</v>
@@ -3035,20 +2966,20 @@
     </row>
     <row r="103" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A103">
-        <v>50</v>
+        <v>70</v>
       </c>
       <c r="B103" t="s">
-        <v>11</v>
+        <v>30</v>
       </c>
       <c r="C103" t="str">
         <f t="shared" si="1"/>
-        <v>EB-P3400XUEGEU</v>
+        <v>178236</v>
       </c>
       <c r="D103" s="3">
-        <v>8806094682748</v>
+        <v>4023103254145</v>
       </c>
       <c r="E103">
-        <v>16</v>
+        <v>155</v>
       </c>
       <c r="F103" t="s">
         <v>6</v>
@@ -3056,20 +2987,19 @@
     </row>
     <row r="104" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A104">
-        <v>5</v>
+        <v>75</v>
       </c>
       <c r="B104" t="s">
-        <v>24</v>
-      </c>
-      <c r="C104" t="str">
-        <f t="shared" si="1"/>
-        <v>SM-L310NZGAEUE</v>
+        <v>31</v>
+      </c>
+      <c r="C104" s="5" t="s">
+        <v>18</v>
       </c>
       <c r="D104" s="3">
-        <v>8806095660981</v>
+        <v>4023103246584</v>
       </c>
       <c r="E104">
-        <v>126</v>
+        <v>17</v>
       </c>
       <c r="F104" t="s">
         <v>6</v>
@@ -3077,191 +3007,191 @@
     </row>
     <row r="105" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A105">
-        <v>15</v>
+        <v>95</v>
       </c>
       <c r="B105" t="s">
-        <v>25</v>
+        <v>49</v>
       </c>
       <c r="C105" t="str">
         <f t="shared" si="1"/>
-        <v>SM-L320NZSAEUE</v>
+        <v>BHR6151DE</v>
       </c>
       <c r="D105" s="3">
-        <v>8806097415756</v>
+        <v>6934177787782</v>
       </c>
       <c r="E105">
-        <v>165</v>
+        <v>359</v>
       </c>
       <c r="F105" t="s">
-        <v>6</v>
+        <v>122</v>
       </c>
     </row>
     <row r="106" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A106">
-        <v>5</v>
+        <v>300</v>
       </c>
       <c r="B106" t="s">
-        <v>58</v>
+        <v>12</v>
       </c>
       <c r="C106" t="str">
         <f t="shared" si="1"/>
-        <v>S6003EU</v>
+        <v>BHR6942EU</v>
       </c>
       <c r="D106" s="3">
-        <v>622356220743</v>
+        <v>6941812708347</v>
       </c>
       <c r="E106">
-        <v>69</v>
+        <v>49</v>
       </c>
       <c r="F106" t="s">
-        <v>145</v>
+        <v>122</v>
       </c>
     </row>
     <row r="107" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A107">
-        <v>230</v>
+        <v>20</v>
       </c>
       <c r="B107" t="s">
-        <v>84</v>
+        <v>57</v>
       </c>
       <c r="C107" t="str">
         <f t="shared" si="1"/>
-        <v>DT8270E1</v>
+        <v>ELA5956EU</v>
       </c>
       <c r="D107" s="3">
-        <v>3121040084175</v>
+        <v>6941948705630</v>
       </c>
       <c r="E107">
-        <v>34</v>
+        <v>210</v>
       </c>
       <c r="F107" t="s">
-        <v>145</v>
+        <v>122</v>
       </c>
     </row>
     <row r="108" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A108">
-        <v>160</v>
+        <v>4000</v>
       </c>
       <c r="B108" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C108" t="str">
         <f t="shared" si="1"/>
-        <v>FV2835E0</v>
+        <v>PFJ4191EU</v>
       </c>
       <c r="D108" s="3">
-        <v>3121040082201</v>
+        <v>6941948704916</v>
       </c>
       <c r="E108">
-        <v>20</v>
+        <v>41</v>
       </c>
       <c r="F108" t="s">
-        <v>145</v>
+        <v>6</v>
       </c>
     </row>
     <row r="109" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A109">
-        <v>80</v>
+        <v>10</v>
       </c>
       <c r="B109" t="s">
-        <v>92</v>
+        <v>26</v>
       </c>
       <c r="C109" t="str">
         <f t="shared" si="1"/>
-        <v>SV8130E0</v>
+        <v>BHR08OLGL</v>
       </c>
       <c r="D109" s="3">
-        <v>3121040086193</v>
+        <v>6932554471880</v>
       </c>
       <c r="E109">
-        <v>99</v>
+        <v>16</v>
       </c>
       <c r="F109" t="s">
-        <v>145</v>
+        <v>6</v>
       </c>
     </row>
     <row r="110" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A110">
-        <v>45</v>
+        <v>30</v>
       </c>
       <c r="B110" t="s">
-        <v>59</v>
+        <v>27</v>
       </c>
       <c r="C110" t="str">
         <f t="shared" si="1"/>
-        <v>FV6812E0</v>
+        <v>BHR07PSGL</v>
       </c>
       <c r="D110" s="3">
-        <v>3121040077184</v>
+        <v>6932554419813</v>
       </c>
       <c r="E110">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="F110" t="s">
-        <v>145</v>
+        <v>6</v>
       </c>
     </row>
     <row r="111" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A111">
-        <v>20</v>
+        <v>50</v>
       </c>
       <c r="B111" t="s">
-        <v>85</v>
+        <v>62</v>
       </c>
       <c r="C111" t="str">
         <f t="shared" si="1"/>
-        <v>FV8066E0</v>
+        <v>BHR9341GL</v>
       </c>
       <c r="D111" s="3">
-        <v>3121040086490</v>
+        <v>6941812774717</v>
       </c>
       <c r="E111">
-        <v>48</v>
+        <v>17</v>
       </c>
       <c r="F111" t="s">
-        <v>145</v>
+        <v>6</v>
       </c>
     </row>
     <row r="112" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A112">
-        <v>5</v>
+        <v>50</v>
       </c>
       <c r="B112" t="s">
-        <v>86</v>
+        <v>63</v>
       </c>
       <c r="C112" t="str">
         <f t="shared" si="1"/>
-        <v>FV8042E0</v>
+        <v>BHR9333GL</v>
       </c>
       <c r="D112" s="3">
-        <v>3121040086469</v>
+        <v>6941812743669</v>
       </c>
       <c r="E112">
-        <v>48</v>
+        <v>17</v>
       </c>
       <c r="F112" t="s">
-        <v>145</v>
+        <v>6</v>
       </c>
     </row>
     <row r="113" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A113">
-        <v>15</v>
+        <v>40</v>
       </c>
       <c r="B113" t="s">
-        <v>87</v>
+        <v>64</v>
       </c>
       <c r="C113" t="str">
         <f t="shared" si="1"/>
-        <v>FV9E50E0</v>
+        <v>BHR08O7GL</v>
       </c>
       <c r="D113" s="3">
-        <v>3121040089040</v>
+        <v>6932554471200</v>
       </c>
       <c r="E113">
-        <v>93</v>
+        <v>25</v>
       </c>
       <c r="F113" t="s">
-        <v>145</v>
+        <v>6</v>
       </c>
     </row>
     <row r="114" spans="1:6" x14ac:dyDescent="0.25">
@@ -3269,80 +3199,80 @@
         <v>5</v>
       </c>
       <c r="B114" t="s">
-        <v>93</v>
+        <v>28</v>
       </c>
       <c r="C114" t="str">
         <f t="shared" si="1"/>
-        <v>FV5718E0</v>
+        <v>BHR08PLGL</v>
       </c>
       <c r="D114" s="3">
-        <v>3121040075692</v>
+        <v>6932554473877</v>
       </c>
       <c r="E114">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="F114" t="s">
-        <v>145</v>
+        <v>6</v>
       </c>
     </row>
     <row r="115" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A115">
-        <v>5</v>
+        <v>80</v>
       </c>
       <c r="B115" t="s">
-        <v>88</v>
+        <v>7</v>
       </c>
       <c r="C115" t="str">
         <f t="shared" si="1"/>
-        <v>FV6872E0</v>
+        <v>QBH4380GL</v>
       </c>
       <c r="D115" s="3">
-        <v>3121040080184</v>
+        <v>6941948709218</v>
       </c>
       <c r="E115">
-        <v>40</v>
+        <v>12</v>
       </c>
       <c r="F115" t="s">
-        <v>145</v>
+        <v>6</v>
       </c>
     </row>
     <row r="116" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A116">
-        <v>45</v>
+        <v>100</v>
       </c>
       <c r="B116" t="s">
-        <v>122</v>
+        <v>8</v>
       </c>
       <c r="C116" t="str">
         <f t="shared" si="1"/>
-        <v>FV1713</v>
+        <v>QBH4378GL</v>
       </c>
       <c r="D116" s="3">
-        <v>3121040067741</v>
+        <v>6941948709201</v>
       </c>
       <c r="E116">
-        <v>12.430000000000001</v>
+        <v>12</v>
       </c>
       <c r="F116" t="s">
-        <v>145</v>
+        <v>6</v>
       </c>
     </row>
     <row r="117" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A117">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="B117" t="s">
-        <v>89</v>
+        <v>35</v>
       </c>
       <c r="C117" t="str">
         <f t="shared" si="1"/>
-        <v>BC50D4V0</v>
+        <v>QBH4265GL</v>
       </c>
       <c r="D117" s="3">
-        <v>3121040092439</v>
+        <v>6941948702042</v>
       </c>
       <c r="E117">
-        <v>13</v>
+        <v>27</v>
       </c>
       <c r="F117" t="s">
         <v>6</v>
@@ -3350,20 +3280,20 @@
     </row>
     <row r="118" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A118">
-        <v>20</v>
+        <v>60</v>
       </c>
       <c r="B118" t="s">
-        <v>90</v>
+        <v>36</v>
       </c>
       <c r="C118" t="str">
         <f t="shared" si="1"/>
-        <v>PP1803V0</v>
+        <v>QBH4263GL</v>
       </c>
       <c r="D118" s="3">
-        <v>3121040095317</v>
+        <v>6941948702035</v>
       </c>
       <c r="E118">
-        <v>10</v>
+        <v>27</v>
       </c>
       <c r="F118" t="s">
         <v>6</v>
@@ -3371,20 +3301,20 @@
     </row>
     <row r="119" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A119">
-        <v>20</v>
+        <v>40</v>
       </c>
       <c r="B119" t="s">
-        <v>91</v>
+        <v>9</v>
       </c>
       <c r="C119" t="str">
         <f t="shared" si="1"/>
-        <v>PP1806</v>
+        <v>QBH2475GL</v>
       </c>
       <c r="D119" s="3">
-        <v>3121040095355</v>
+        <v>6941948703391</v>
       </c>
       <c r="E119">
-        <v>10</v>
+        <v>38</v>
       </c>
       <c r="F119" t="s">
         <v>6</v>
@@ -3392,20 +3322,20 @@
     </row>
     <row r="120" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A120">
-        <v>70</v>
+        <v>35</v>
       </c>
       <c r="B120" t="s">
-        <v>32</v>
+        <v>58</v>
       </c>
       <c r="C120" t="str">
         <f t="shared" si="1"/>
-        <v>178236</v>
+        <v>BHR9036EU</v>
       </c>
       <c r="D120" s="3">
-        <v>4023103254145</v>
+        <v>6941812797013</v>
       </c>
       <c r="E120">
-        <v>155</v>
+        <v>17</v>
       </c>
       <c r="F120" t="s">
         <v>6</v>
@@ -3413,19 +3343,20 @@
     </row>
     <row r="121" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A121">
-        <v>80</v>
+        <v>40</v>
       </c>
       <c r="B121" t="s">
-        <v>33</v>
-      </c>
-      <c r="C121" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="C121" t="str">
+        <f t="shared" si="1"/>
+        <v>BHR8811EU</v>
+      </c>
+      <c r="D121" s="3">
+        <v>6941812791868</v>
+      </c>
+      <c r="E121">
         <v>18</v>
-      </c>
-      <c r="D121" s="3">
-        <v>4023103246584</v>
-      </c>
-      <c r="E121">
-        <v>17</v>
       </c>
       <c r="F121" t="s">
         <v>6</v>
@@ -3433,526 +3364,43 @@
     </row>
     <row r="122" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A122">
-        <v>120</v>
+        <v>5</v>
       </c>
       <c r="B122" t="s">
-        <v>54</v>
+        <v>25</v>
       </c>
       <c r="C122" t="str">
         <f t="shared" si="1"/>
-        <v>BHR6151DE</v>
+        <v>BHR5967EU</v>
       </c>
       <c r="D122" s="3">
-        <v>6934177787782</v>
+        <v>6934177763113</v>
       </c>
       <c r="E122">
-        <v>349</v>
+        <v>28</v>
       </c>
       <c r="F122" t="s">
-        <v>145</v>
+        <v>6</v>
       </c>
     </row>
     <row r="123" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A123">
-        <v>300</v>
+        <v>40</v>
       </c>
       <c r="B123" t="s">
-        <v>12</v>
+        <v>59</v>
       </c>
       <c r="C123" t="str">
         <f t="shared" si="1"/>
-        <v>BHR6942EU</v>
+        <v>BHR9099GL</v>
       </c>
       <c r="D123" s="3">
-        <v>6941812708347</v>
+        <v>6941812797853</v>
       </c>
       <c r="E123">
-        <v>49</v>
+        <v>39</v>
       </c>
       <c r="F123" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="124" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A124">
-        <v>15</v>
-      </c>
-      <c r="B124" t="s">
-        <v>68</v>
-      </c>
-      <c r="C124" t="str">
-        <f t="shared" si="1"/>
-        <v>BHR5274GL</v>
-      </c>
-      <c r="D124" s="3">
-        <v>6934177751158</v>
-      </c>
-      <c r="E124">
-        <v>95</v>
-      </c>
-      <c r="F124" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="125" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A125">
-        <v>15</v>
-      </c>
-      <c r="B125" t="s">
-        <v>69</v>
-      </c>
-      <c r="C125" t="str">
-        <f t="shared" si="1"/>
-        <v>BHR08MZEU</v>
-      </c>
-      <c r="D125" s="3">
-        <v>6932554469139</v>
-      </c>
-      <c r="E125">
-        <v>123</v>
-      </c>
-      <c r="F125" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="126" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A126">
-        <v>50</v>
-      </c>
-      <c r="B126" t="s">
-        <v>146</v>
-      </c>
-      <c r="C126" t="str">
-        <f t="shared" ref="C126:C146" si="2">MID(B126,FIND("@",SUBSTITUTE(B126," ","@",LEN(B126)-LEN(SUBSTITUTE(B126," ",""))))+1,LEN(B126))</f>
-        <v>BHR084AEU</v>
-      </c>
-      <c r="D126" s="3">
-        <v>6932554440893</v>
-      </c>
-      <c r="E126">
-        <v>102</v>
-      </c>
-      <c r="F126" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="127" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A127">
-        <v>15</v>
-      </c>
-      <c r="B127" t="s">
-        <v>26</v>
-      </c>
-      <c r="C127" t="str">
-        <f t="shared" si="2"/>
-        <v>BHR9798EU</v>
-      </c>
-      <c r="D127" s="3">
-        <v>6932554403850</v>
-      </c>
-      <c r="E127">
-        <v>59</v>
-      </c>
-      <c r="F127" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="128" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A128">
-        <v>30</v>
-      </c>
-      <c r="B128" t="s">
-        <v>70</v>
-      </c>
-      <c r="C128" t="str">
-        <f t="shared" si="2"/>
-        <v>ELA5956EU</v>
-      </c>
-      <c r="D128" s="3">
-        <v>6941948705630</v>
-      </c>
-      <c r="E128">
-        <v>210</v>
-      </c>
-      <c r="F128" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="129" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A129">
-        <v>4000</v>
-      </c>
-      <c r="B129" t="s">
-        <v>76</v>
-      </c>
-      <c r="C129" t="str">
-        <f t="shared" si="2"/>
-        <v>PFJ4191EU</v>
-      </c>
-      <c r="D129" s="3">
-        <v>6941948704916</v>
-      </c>
-      <c r="E129">
-        <v>41</v>
-      </c>
-      <c r="F129" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="130" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A130">
-        <v>10</v>
-      </c>
-      <c r="B130" t="s">
-        <v>28</v>
-      </c>
-      <c r="C130" t="str">
-        <f t="shared" si="2"/>
-        <v>BHR08OLGL</v>
-      </c>
-      <c r="D130" s="3">
-        <v>6932554471880</v>
-      </c>
-      <c r="E130">
-        <v>16</v>
-      </c>
-      <c r="F130" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="131" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A131">
-        <v>30</v>
-      </c>
-      <c r="B131" t="s">
-        <v>29</v>
-      </c>
-      <c r="C131" t="str">
-        <f t="shared" si="2"/>
-        <v>BHR07PSGL</v>
-      </c>
-      <c r="D131" s="3">
-        <v>6932554419813</v>
-      </c>
-      <c r="E131">
-        <v>30</v>
-      </c>
-      <c r="F131" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="132" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A132">
-        <v>60</v>
-      </c>
-      <c r="B132" t="s">
-        <v>77</v>
-      </c>
-      <c r="C132" t="str">
-        <f t="shared" si="2"/>
-        <v>BHR9341GL</v>
-      </c>
-      <c r="D132" s="3">
-        <v>6941812774717</v>
-      </c>
-      <c r="E132">
-        <v>17</v>
-      </c>
-      <c r="F132" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="133" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A133">
-        <v>60</v>
-      </c>
-      <c r="B133" t="s">
-        <v>78</v>
-      </c>
-      <c r="C133" t="str">
-        <f t="shared" si="2"/>
-        <v>BHR9333GL</v>
-      </c>
-      <c r="D133" s="3">
-        <v>6941812743669</v>
-      </c>
-      <c r="E133">
-        <v>17</v>
-      </c>
-      <c r="F133" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="134" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A134">
-        <v>40</v>
-      </c>
-      <c r="B134" t="s">
-        <v>79</v>
-      </c>
-      <c r="C134" t="str">
-        <f t="shared" si="2"/>
-        <v>BHR08O7GL</v>
-      </c>
-      <c r="D134" s="3">
-        <v>6932554471200</v>
-      </c>
-      <c r="E134">
-        <v>25</v>
-      </c>
-      <c r="F134" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="135" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A135">
-        <v>5</v>
-      </c>
-      <c r="B135" t="s">
-        <v>30</v>
-      </c>
-      <c r="C135" t="str">
-        <f t="shared" si="2"/>
-        <v>BHR08PLGL</v>
-      </c>
-      <c r="D135" s="3">
-        <v>6932554473877</v>
-      </c>
-      <c r="E135">
-        <v>20</v>
-      </c>
-      <c r="F135" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="136" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A136">
-        <v>80</v>
-      </c>
-      <c r="B136" t="s">
-        <v>7</v>
-      </c>
-      <c r="C136" t="str">
-        <f t="shared" si="2"/>
-        <v>QBH4380GL</v>
-      </c>
-      <c r="D136" s="3">
-        <v>6941948709218</v>
-      </c>
-      <c r="E136">
-        <v>12</v>
-      </c>
-      <c r="F136" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="137" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A137">
-        <v>100</v>
-      </c>
-      <c r="B137" t="s">
-        <v>8</v>
-      </c>
-      <c r="C137" t="str">
-        <f t="shared" si="2"/>
-        <v>QBH4378GL</v>
-      </c>
-      <c r="D137" s="3">
-        <v>6941948709201</v>
-      </c>
-      <c r="E137">
-        <v>12</v>
-      </c>
-      <c r="F137" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="138" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A138">
-        <v>40</v>
-      </c>
-      <c r="B138" t="s">
-        <v>38</v>
-      </c>
-      <c r="C138" t="str">
-        <f t="shared" si="2"/>
-        <v>QBH4265GL</v>
-      </c>
-      <c r="D138" s="3">
-        <v>6941948702042</v>
-      </c>
-      <c r="E138">
-        <v>27</v>
-      </c>
-      <c r="F138" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="139" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A139">
-        <v>5</v>
-      </c>
-      <c r="B139" t="s">
-        <v>39</v>
-      </c>
-      <c r="C139" t="str">
-        <f t="shared" si="2"/>
-        <v>QBH4370GL</v>
-      </c>
-      <c r="D139" s="3">
-        <v>6941948709164</v>
-      </c>
-      <c r="E139">
-        <v>27</v>
-      </c>
-      <c r="F139" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="140" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A140">
-        <v>5</v>
-      </c>
-      <c r="B140" t="s">
-        <v>40</v>
-      </c>
-      <c r="C140" t="str">
-        <f t="shared" si="2"/>
-        <v>QBH4372GL</v>
-      </c>
-      <c r="D140" s="3">
-        <v>6941948709171</v>
-      </c>
-      <c r="E140">
-        <v>27</v>
-      </c>
-      <c r="F140" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="141" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A141">
-        <v>70</v>
-      </c>
-      <c r="B141" t="s">
-        <v>41</v>
-      </c>
-      <c r="C141" t="str">
-        <f t="shared" si="2"/>
-        <v>QBH4263GL</v>
-      </c>
-      <c r="D141" s="3">
-        <v>6941948702035</v>
-      </c>
-      <c r="E141">
-        <v>27</v>
-      </c>
-      <c r="F141" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="142" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A142">
-        <v>50</v>
-      </c>
-      <c r="B142" t="s">
-        <v>9</v>
-      </c>
-      <c r="C142" t="str">
-        <f t="shared" si="2"/>
-        <v>QBH2475GL</v>
-      </c>
-      <c r="D142" s="3">
-        <v>6941948703391</v>
-      </c>
-      <c r="E142">
-        <v>38</v>
-      </c>
-      <c r="F142" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="143" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A143">
-        <v>40</v>
-      </c>
-      <c r="B143" t="s">
-        <v>71</v>
-      </c>
-      <c r="C143" t="str">
-        <f t="shared" si="2"/>
-        <v>BHR9036EU</v>
-      </c>
-      <c r="D143" s="3">
-        <v>6941812797013</v>
-      </c>
-      <c r="E143">
-        <v>17</v>
-      </c>
-      <c r="F143" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="144" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A144">
-        <v>40</v>
-      </c>
-      <c r="B144" t="s">
-        <v>13</v>
-      </c>
-      <c r="C144" t="str">
-        <f t="shared" si="2"/>
-        <v>BHR8811EU</v>
-      </c>
-      <c r="D144" s="3">
-        <v>6941812791868</v>
-      </c>
-      <c r="E144">
-        <v>18</v>
-      </c>
-      <c r="F144" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="145" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A145">
-        <v>10</v>
-      </c>
-      <c r="B145" t="s">
-        <v>27</v>
-      </c>
-      <c r="C145" t="str">
-        <f t="shared" si="2"/>
-        <v>BHR5967EU</v>
-      </c>
-      <c r="D145" s="3">
-        <v>6934177763113</v>
-      </c>
-      <c r="E145">
-        <v>28</v>
-      </c>
-      <c r="F145" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="146" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A146">
-        <v>40</v>
-      </c>
-      <c r="B146" t="s">
-        <v>72</v>
-      </c>
-      <c r="C146" t="str">
-        <f t="shared" si="2"/>
-        <v>BHR9099GL</v>
-      </c>
-      <c r="D146" s="3">
-        <v>6941812797853</v>
-      </c>
-      <c r="E146">
-        <v>39</v>
-      </c>
-      <c r="F146" t="s">
         <v>6</v>
       </c>
     </row>

</xml_diff>